<commit_message>
Add data file for sail size recommendations
</commit_message>
<xml_diff>
--- a/data/research.xlsx
+++ b/data/research.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ninal\Desktop\projects\Julia Project\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ninal\Desktop\projects\NinasProject\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE2E856F-3C61-4F70-9B36-40F458C9AA85}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3A8F283-A286-4E3C-8185-A2373BCFE143}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="21585" windowHeight="8820" xr2:uid="{9C4ED264-3AF9-4DAD-A95C-E7848EE8F76F}"/>
   </bookViews>
@@ -259,7 +259,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -308,35 +308,41 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -653,208 +659,215 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3B9AD222-34BA-409C-82CD-7E525C4015EB}">
-  <dimension ref="A1:AM29"/>
+  <dimension ref="A1:AN29"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="13.15" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="15.19921875" style="3" customWidth="1"/>
-    <col min="2" max="34" width="3.73046875" style="3" customWidth="1"/>
-    <col min="35" max="35" width="2.53125" style="3" customWidth="1"/>
-    <col min="36" max="16384" width="10.6640625" style="3"/>
+    <col min="2" max="36" width="3.59765625" style="3" customWidth="1"/>
+    <col min="37" max="16384" width="10.6640625" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:39" ht="14.25" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:40" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A1" s="23" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="2" spans="1:39" x14ac:dyDescent="0.4">
+      <c r="B1" s="23"/>
+    </row>
+    <row r="2" spans="1:40" x14ac:dyDescent="0.4">
       <c r="A2" s="21" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="3" spans="1:39" x14ac:dyDescent="0.4">
+      <c r="B2" s="21"/>
+    </row>
+    <row r="3" spans="1:40" x14ac:dyDescent="0.4">
       <c r="A3" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="26">
+      <c r="B3" s="24">
+        <v>0</v>
+      </c>
+      <c r="C3" s="26">
         <v>1</v>
       </c>
-      <c r="C3" s="26"/>
       <c r="D3" s="26"/>
-      <c r="E3" s="26">
+      <c r="E3" s="26"/>
+      <c r="F3" s="26">
         <v>2</v>
       </c>
-      <c r="F3" s="26"/>
       <c r="G3" s="26"/>
-      <c r="H3" s="26">
+      <c r="H3" s="26"/>
+      <c r="I3" s="26">
         <v>3</v>
       </c>
-      <c r="I3" s="26"/>
       <c r="J3" s="26"/>
       <c r="K3" s="26"/>
-      <c r="L3" s="26">
+      <c r="L3" s="26"/>
+      <c r="M3" s="26">
         <v>4</v>
       </c>
-      <c r="M3" s="26"/>
       <c r="N3" s="26"/>
       <c r="O3" s="26"/>
       <c r="P3" s="26"/>
       <c r="Q3" s="26"/>
-      <c r="R3" s="26">
+      <c r="R3" s="26"/>
+      <c r="S3" s="26">
         <v>5</v>
       </c>
-      <c r="S3" s="26"/>
       <c r="T3" s="26"/>
       <c r="U3" s="26"/>
       <c r="V3" s="26"/>
-      <c r="W3" s="26">
+      <c r="W3" s="26"/>
+      <c r="X3" s="26">
         <v>6</v>
       </c>
-      <c r="X3" s="26"/>
       <c r="Y3" s="26"/>
       <c r="Z3" s="26"/>
       <c r="AA3" s="26"/>
       <c r="AB3" s="26"/>
-      <c r="AC3" s="26">
+      <c r="AC3" s="26"/>
+      <c r="AD3" s="26">
         <v>7</v>
       </c>
-      <c r="AD3" s="26"/>
       <c r="AE3" s="26"/>
       <c r="AF3" s="26"/>
       <c r="AG3" s="26"/>
       <c r="AH3" s="26"/>
-      <c r="AJ3" s="8" t="s">
+      <c r="AI3" s="26"/>
+      <c r="AK3" s="8" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:39" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:40" x14ac:dyDescent="0.4">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="2">
+      <c r="B4" s="24">
+        <v>0</v>
+      </c>
+      <c r="C4" s="2">
         <v>1</v>
       </c>
-      <c r="C4" s="2">
+      <c r="D4" s="2">
         <v>2</v>
       </c>
-      <c r="D4" s="2">
+      <c r="E4" s="2">
         <v>3</v>
       </c>
-      <c r="E4" s="2">
+      <c r="F4" s="2">
         <v>4</v>
       </c>
-      <c r="F4" s="2">
+      <c r="G4" s="2">
         <v>5</v>
       </c>
-      <c r="G4" s="2">
+      <c r="H4" s="2">
         <v>6</v>
       </c>
-      <c r="H4" s="2">
+      <c r="I4" s="2">
         <v>7</v>
       </c>
-      <c r="I4" s="2">
+      <c r="J4" s="2">
         <v>8</v>
       </c>
-      <c r="J4" s="2">
+      <c r="K4" s="2">
         <v>9</v>
       </c>
-      <c r="K4" s="2">
+      <c r="L4" s="2">
         <v>10</v>
       </c>
-      <c r="L4" s="2">
+      <c r="M4" s="2">
         <v>11</v>
       </c>
-      <c r="M4" s="2">
+      <c r="N4" s="2">
         <v>12</v>
       </c>
-      <c r="N4" s="2">
+      <c r="O4" s="2">
         <v>13</v>
       </c>
-      <c r="O4" s="2">
+      <c r="P4" s="2">
         <v>14</v>
       </c>
-      <c r="P4" s="2">
+      <c r="Q4" s="2">
         <v>15</v>
       </c>
-      <c r="Q4" s="2">
+      <c r="R4" s="2">
         <v>16</v>
       </c>
-      <c r="R4" s="2">
+      <c r="S4" s="2">
         <v>17</v>
       </c>
-      <c r="S4" s="2">
+      <c r="T4" s="2">
         <v>18</v>
       </c>
-      <c r="T4" s="2">
+      <c r="U4" s="2">
         <v>19</v>
       </c>
-      <c r="U4" s="2">
+      <c r="V4" s="2">
         <v>20</v>
       </c>
-      <c r="V4" s="2">
+      <c r="W4" s="2">
         <v>21</v>
       </c>
-      <c r="W4" s="2">
+      <c r="X4" s="2">
         <v>22</v>
       </c>
-      <c r="X4" s="2">
+      <c r="Y4" s="2">
         <v>23</v>
       </c>
-      <c r="Y4" s="2">
+      <c r="Z4" s="2">
         <v>24</v>
       </c>
-      <c r="Z4" s="2">
+      <c r="AA4" s="2">
         <v>25</v>
       </c>
-      <c r="AA4" s="2">
+      <c r="AB4" s="2">
         <v>26</v>
       </c>
-      <c r="AB4" s="2">
+      <c r="AC4" s="2">
         <v>27</v>
       </c>
-      <c r="AC4" s="2">
+      <c r="AD4" s="2">
         <v>28</v>
       </c>
-      <c r="AD4" s="2">
+      <c r="AE4" s="2">
         <v>29</v>
       </c>
-      <c r="AE4" s="2">
+      <c r="AF4" s="2">
         <v>30</v>
       </c>
-      <c r="AF4" s="2">
+      <c r="AG4" s="2">
         <v>31</v>
       </c>
-      <c r="AG4" s="2">
+      <c r="AH4" s="2">
         <v>32</v>
       </c>
-      <c r="AH4" s="2">
+      <c r="AI4" s="2">
         <v>33</v>
       </c>
-      <c r="AJ4" s="9" t="s">
+      <c r="AK4" s="9" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:39" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:40" x14ac:dyDescent="0.4">
       <c r="A5" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="B5" s="33"/>
-      <c r="C5" s="33"/>
-      <c r="D5" s="33"/>
-      <c r="E5" s="32"/>
-      <c r="F5" s="32"/>
-      <c r="G5" s="32"/>
-      <c r="H5" s="31"/>
-      <c r="I5" s="31"/>
-      <c r="J5" s="31"/>
-      <c r="K5" s="31"/>
-      <c r="L5" s="30"/>
+      <c r="B5" s="35"/>
+      <c r="C5" s="25"/>
+      <c r="D5" s="25"/>
+      <c r="E5" s="25"/>
+      <c r="F5" s="27"/>
+      <c r="G5" s="27"/>
+      <c r="H5" s="27"/>
+      <c r="I5" s="28"/>
+      <c r="J5" s="28"/>
+      <c r="K5" s="28"/>
+      <c r="L5" s="28"/>
       <c r="M5" s="30"/>
       <c r="N5" s="30"/>
       <c r="O5" s="30"/>
       <c r="P5" s="30"/>
       <c r="Q5" s="30"/>
-      <c r="R5" s="29"/>
+      <c r="R5" s="30"/>
       <c r="S5" s="29"/>
       <c r="T5" s="29"/>
       <c r="U5" s="29"/>
@@ -871,36 +884,37 @@
       <c r="AF5" s="29"/>
       <c r="AG5" s="29"/>
       <c r="AH5" s="29"/>
-      <c r="AJ5" s="10" t="s">
+      <c r="AI5" s="29"/>
+      <c r="AK5" s="10" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:39" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:40" x14ac:dyDescent="0.4">
       <c r="A6" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="B6" s="33"/>
-      <c r="C6" s="33"/>
-      <c r="D6" s="33"/>
-      <c r="E6" s="33"/>
-      <c r="F6" s="33"/>
-      <c r="G6" s="33"/>
-      <c r="H6" s="32"/>
-      <c r="I6" s="32"/>
-      <c r="J6" s="32"/>
-      <c r="K6" s="32"/>
-      <c r="L6" s="31"/>
-      <c r="M6" s="31"/>
-      <c r="N6" s="31"/>
-      <c r="O6" s="31"/>
-      <c r="P6" s="31"/>
-      <c r="Q6" s="31"/>
-      <c r="R6" s="30"/>
+      <c r="B6" s="35"/>
+      <c r="C6" s="25"/>
+      <c r="D6" s="25"/>
+      <c r="E6" s="25"/>
+      <c r="F6" s="25"/>
+      <c r="G6" s="25"/>
+      <c r="H6" s="25"/>
+      <c r="I6" s="27"/>
+      <c r="J6" s="27"/>
+      <c r="K6" s="27"/>
+      <c r="L6" s="27"/>
+      <c r="M6" s="28"/>
+      <c r="N6" s="28"/>
+      <c r="O6" s="28"/>
+      <c r="P6" s="28"/>
+      <c r="Q6" s="28"/>
+      <c r="R6" s="28"/>
       <c r="S6" s="30"/>
       <c r="T6" s="30"/>
       <c r="U6" s="30"/>
       <c r="V6" s="30"/>
-      <c r="W6" s="29"/>
+      <c r="W6" s="30"/>
       <c r="X6" s="29"/>
       <c r="Y6" s="29"/>
       <c r="Z6" s="29"/>
@@ -912,89 +926,92 @@
       <c r="AF6" s="29"/>
       <c r="AG6" s="29"/>
       <c r="AH6" s="29"/>
-      <c r="AI6" s="5"/>
-      <c r="AJ6" s="11" t="s">
+      <c r="AI6" s="29"/>
+      <c r="AJ6" s="5"/>
+      <c r="AK6" s="11" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="7" spans="1:39" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:40" x14ac:dyDescent="0.4">
       <c r="A7" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="B7" s="33"/>
-      <c r="C7" s="33"/>
-      <c r="D7" s="33"/>
-      <c r="E7" s="33"/>
-      <c r="F7" s="33"/>
-      <c r="G7" s="33"/>
-      <c r="H7" s="32"/>
-      <c r="I7" s="32"/>
-      <c r="J7" s="32"/>
-      <c r="K7" s="32"/>
-      <c r="L7" s="32"/>
-      <c r="M7" s="32"/>
-      <c r="N7" s="32"/>
-      <c r="O7" s="32"/>
-      <c r="P7" s="32"/>
-      <c r="Q7" s="32"/>
-      <c r="R7" s="31"/>
-      <c r="S7" s="31"/>
-      <c r="T7" s="31"/>
-      <c r="U7" s="31"/>
-      <c r="V7" s="31"/>
-      <c r="W7" s="30"/>
+      <c r="B7" s="35"/>
+      <c r="C7" s="25"/>
+      <c r="D7" s="25"/>
+      <c r="E7" s="25"/>
+      <c r="F7" s="25"/>
+      <c r="G7" s="25"/>
+      <c r="H7" s="25"/>
+      <c r="I7" s="27"/>
+      <c r="J7" s="27"/>
+      <c r="K7" s="27"/>
+      <c r="L7" s="27"/>
+      <c r="M7" s="27"/>
+      <c r="N7" s="27"/>
+      <c r="O7" s="27"/>
+      <c r="P7" s="27"/>
+      <c r="Q7" s="27"/>
+      <c r="R7" s="27"/>
+      <c r="S7" s="28"/>
+      <c r="T7" s="28"/>
+      <c r="U7" s="28"/>
+      <c r="V7" s="28"/>
+      <c r="W7" s="28"/>
       <c r="X7" s="30"/>
       <c r="Y7" s="30"/>
       <c r="Z7" s="30"/>
       <c r="AA7" s="30"/>
       <c r="AB7" s="30"/>
-      <c r="AC7" s="29"/>
+      <c r="AC7" s="30"/>
       <c r="AD7" s="29"/>
       <c r="AE7" s="29"/>
       <c r="AF7" s="29"/>
       <c r="AG7" s="29"/>
       <c r="AH7" s="29"/>
-      <c r="AJ7" s="12" t="s">
+      <c r="AI7" s="29"/>
+      <c r="AK7" s="12" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="8" spans="1:39" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:40" x14ac:dyDescent="0.4">
       <c r="A8" s="22" t="s">
         <v>32</v>
       </c>
-      <c r="B8" s="6"/>
+      <c r="B8" s="22"/>
       <c r="C8" s="6"/>
       <c r="D8" s="6"/>
-    </row>
-    <row r="9" spans="1:39" x14ac:dyDescent="0.4">
+      <c r="E8" s="6"/>
+    </row>
+    <row r="9" spans="1:40" x14ac:dyDescent="0.4">
       <c r="A9" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="B9" s="6"/>
+      <c r="B9" s="4"/>
       <c r="C9" s="6"/>
       <c r="D9" s="6"/>
-      <c r="F9" s="6"/>
+      <c r="E9" s="6"/>
       <c r="G9" s="6"/>
-      <c r="H9" s="25" t="s">
+      <c r="H9" s="6"/>
+      <c r="I9" s="31" t="s">
         <v>18</v>
       </c>
-      <c r="I9" s="26"/>
       <c r="J9" s="26"/>
       <c r="K9" s="26"/>
       <c r="L9" s="26"/>
       <c r="M9" s="26"/>
-      <c r="N9" s="25" t="s">
+      <c r="N9" s="26"/>
+      <c r="O9" s="31" t="s">
         <v>12</v>
       </c>
-      <c r="O9" s="26"/>
       <c r="P9" s="26"/>
       <c r="Q9" s="26"/>
       <c r="R9" s="26"/>
       <c r="S9" s="26"/>
-      <c r="T9" s="25" t="s">
+      <c r="T9" s="26"/>
+      <c r="U9" s="31" t="s">
         <v>23</v>
       </c>
-      <c r="U9" s="26"/>
       <c r="V9" s="26"/>
       <c r="W9" s="26"/>
       <c r="X9" s="26"/>
@@ -1002,46 +1019,47 @@
       <c r="Z9" s="26"/>
       <c r="AA9" s="26"/>
       <c r="AB9" s="26"/>
-      <c r="AC9" s="14" t="s">
+      <c r="AC9" s="26"/>
+      <c r="AD9" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="AD9" s="14"/>
       <c r="AE9" s="14"/>
       <c r="AF9" s="14"/>
       <c r="AG9" s="14"/>
       <c r="AH9" s="14"/>
-      <c r="AJ9" s="18"/>
-    </row>
-    <row r="10" spans="1:39" x14ac:dyDescent="0.4">
+      <c r="AI9" s="14"/>
+      <c r="AK9" s="18"/>
+    </row>
+    <row r="10" spans="1:40" x14ac:dyDescent="0.4">
       <c r="A10" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="B10" s="6"/>
+      <c r="B10" s="4"/>
       <c r="C10" s="6"/>
       <c r="D10" s="6"/>
-      <c r="E10" s="17"/>
-      <c r="F10" s="6"/>
+      <c r="E10" s="6"/>
+      <c r="F10" s="17"/>
       <c r="G10" s="6"/>
-      <c r="H10" s="25" t="s">
+      <c r="H10" s="6"/>
+      <c r="I10" s="31" t="s">
         <v>19</v>
       </c>
-      <c r="I10" s="26"/>
       <c r="J10" s="26"/>
       <c r="K10" s="26"/>
       <c r="L10" s="26"/>
       <c r="M10" s="26"/>
-      <c r="N10" s="25" t="s">
+      <c r="N10" s="26"/>
+      <c r="O10" s="31" t="s">
         <v>18</v>
       </c>
-      <c r="O10" s="26"/>
       <c r="P10" s="26"/>
       <c r="Q10" s="26"/>
       <c r="R10" s="26"/>
       <c r="S10" s="26"/>
-      <c r="T10" s="26" t="s">
+      <c r="T10" s="26"/>
+      <c r="U10" s="26" t="s">
         <v>12</v>
       </c>
-      <c r="U10" s="26"/>
       <c r="V10" s="26"/>
       <c r="W10" s="26"/>
       <c r="X10" s="26"/>
@@ -1049,49 +1067,50 @@
       <c r="Z10" s="26"/>
       <c r="AA10" s="26"/>
       <c r="AB10" s="26"/>
-      <c r="AC10" s="14" t="s">
+      <c r="AC10" s="26"/>
+      <c r="AD10" s="14" t="s">
         <v>27</v>
       </c>
-      <c r="AD10" s="14"/>
       <c r="AE10" s="14"/>
       <c r="AF10" s="14"/>
       <c r="AG10" s="14"/>
       <c r="AH10" s="14"/>
-      <c r="AJ10" s="15"/>
-      <c r="AK10" s="13"/>
+      <c r="AI10" s="14"/>
+      <c r="AK10" s="15"/>
       <c r="AL10" s="13"/>
       <c r="AM10" s="13"/>
-    </row>
-    <row r="11" spans="1:39" x14ac:dyDescent="0.4">
+      <c r="AN10" s="13"/>
+    </row>
+    <row r="11" spans="1:40" x14ac:dyDescent="0.4">
       <c r="A11" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B11" s="6"/>
+      <c r="B11" s="4"/>
       <c r="C11" s="6"/>
       <c r="D11" s="6"/>
-      <c r="E11" s="17"/>
-      <c r="F11" s="6"/>
+      <c r="E11" s="6"/>
+      <c r="F11" s="17"/>
       <c r="G11" s="6"/>
-      <c r="H11" s="25" t="s">
+      <c r="H11" s="6"/>
+      <c r="I11" s="31" t="s">
         <v>13</v>
       </c>
-      <c r="I11" s="26"/>
       <c r="J11" s="26"/>
       <c r="K11" s="26"/>
       <c r="L11" s="26"/>
       <c r="M11" s="26"/>
-      <c r="N11" s="25" t="s">
+      <c r="N11" s="26"/>
+      <c r="O11" s="31" t="s">
         <v>19</v>
       </c>
-      <c r="O11" s="26"/>
       <c r="P11" s="26"/>
       <c r="Q11" s="26"/>
       <c r="R11" s="26"/>
       <c r="S11" s="26"/>
-      <c r="T11" s="26" t="s">
+      <c r="T11" s="26"/>
+      <c r="U11" s="26" t="s">
         <v>18</v>
       </c>
-      <c r="U11" s="26"/>
       <c r="V11" s="26"/>
       <c r="W11" s="26"/>
       <c r="X11" s="26"/>
@@ -1099,46 +1118,47 @@
       <c r="Z11" s="26"/>
       <c r="AA11" s="26"/>
       <c r="AB11" s="26"/>
-      <c r="AC11" s="14" t="s">
+      <c r="AC11" s="26"/>
+      <c r="AD11" s="14" t="s">
         <v>28</v>
       </c>
-      <c r="AD11" s="14"/>
       <c r="AE11" s="14"/>
       <c r="AF11" s="14"/>
       <c r="AG11" s="14"/>
       <c r="AH11" s="14"/>
-      <c r="AJ11" s="15"/>
-    </row>
-    <row r="12" spans="1:39" x14ac:dyDescent="0.4">
+      <c r="AI11" s="14"/>
+      <c r="AK11" s="15"/>
+    </row>
+    <row r="12" spans="1:40" x14ac:dyDescent="0.4">
       <c r="A12" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="B12" s="6"/>
+      <c r="B12" s="4"/>
       <c r="C12" s="6"/>
       <c r="D12" s="6"/>
-      <c r="E12" s="17"/>
-      <c r="F12" s="6"/>
+      <c r="E12" s="6"/>
+      <c r="F12" s="17"/>
       <c r="G12" s="6"/>
-      <c r="H12" s="27" t="s">
+      <c r="H12" s="6"/>
+      <c r="I12" s="33" t="s">
         <v>21</v>
       </c>
-      <c r="I12" s="28"/>
-      <c r="J12" s="28"/>
-      <c r="K12" s="28"/>
-      <c r="L12" s="28"/>
-      <c r="M12" s="28"/>
-      <c r="N12" s="25" t="s">
+      <c r="J12" s="34"/>
+      <c r="K12" s="34"/>
+      <c r="L12" s="34"/>
+      <c r="M12" s="34"/>
+      <c r="N12" s="34"/>
+      <c r="O12" s="31" t="s">
         <v>13</v>
       </c>
-      <c r="O12" s="26"/>
       <c r="P12" s="26"/>
       <c r="Q12" s="26"/>
       <c r="R12" s="26"/>
       <c r="S12" s="26"/>
-      <c r="T12" s="26" t="s">
+      <c r="T12" s="26"/>
+      <c r="U12" s="26" t="s">
         <v>19</v>
       </c>
-      <c r="U12" s="26"/>
       <c r="V12" s="26"/>
       <c r="W12" s="26"/>
       <c r="X12" s="26"/>
@@ -1146,46 +1166,47 @@
       <c r="Z12" s="26"/>
       <c r="AA12" s="26"/>
       <c r="AB12" s="26"/>
-      <c r="AC12" s="14" t="s">
+      <c r="AC12" s="26"/>
+      <c r="AD12" s="14" t="s">
         <v>29</v>
       </c>
-      <c r="AD12" s="14"/>
       <c r="AE12" s="14"/>
       <c r="AF12" s="14"/>
       <c r="AG12" s="14"/>
       <c r="AH12" s="14"/>
-      <c r="AJ12" s="15"/>
-    </row>
-    <row r="13" spans="1:39" x14ac:dyDescent="0.4">
+      <c r="AI12" s="14"/>
+      <c r="AK12" s="15"/>
+    </row>
+    <row r="13" spans="1:40" x14ac:dyDescent="0.4">
       <c r="A13" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="B13" s="6"/>
+      <c r="B13" s="4"/>
       <c r="C13" s="6"/>
       <c r="D13" s="6"/>
-      <c r="E13" s="17"/>
-      <c r="F13" s="6"/>
+      <c r="E13" s="6"/>
+      <c r="F13" s="17"/>
       <c r="G13" s="6"/>
-      <c r="H13" s="27" t="s">
+      <c r="H13" s="6"/>
+      <c r="I13" s="33" t="s">
         <v>22</v>
       </c>
-      <c r="I13" s="28"/>
-      <c r="J13" s="28"/>
-      <c r="K13" s="28"/>
-      <c r="L13" s="28"/>
-      <c r="M13" s="28"/>
-      <c r="N13" s="25" t="s">
+      <c r="J13" s="34"/>
+      <c r="K13" s="34"/>
+      <c r="L13" s="34"/>
+      <c r="M13" s="34"/>
+      <c r="N13" s="34"/>
+      <c r="O13" s="31" t="s">
         <v>21</v>
       </c>
-      <c r="O13" s="26"/>
       <c r="P13" s="26"/>
       <c r="Q13" s="26"/>
       <c r="R13" s="26"/>
       <c r="S13" s="26"/>
-      <c r="T13" s="26" t="s">
+      <c r="T13" s="26"/>
+      <c r="U13" s="26" t="s">
         <v>13</v>
       </c>
-      <c r="U13" s="26"/>
       <c r="V13" s="26"/>
       <c r="W13" s="26"/>
       <c r="X13" s="26"/>
@@ -1193,49 +1214,50 @@
       <c r="Z13" s="26"/>
       <c r="AA13" s="26"/>
       <c r="AB13" s="26"/>
-      <c r="AC13" s="14" t="s">
+      <c r="AC13" s="26"/>
+      <c r="AD13" s="14" t="s">
         <v>30</v>
       </c>
-      <c r="AD13" s="14"/>
       <c r="AE13" s="14"/>
       <c r="AF13" s="14"/>
       <c r="AG13" s="14"/>
       <c r="AH13" s="14"/>
-      <c r="AJ13" s="15"/>
-      <c r="AK13" s="13"/>
+      <c r="AI13" s="14"/>
+      <c r="AK13" s="15"/>
       <c r="AL13" s="13"/>
       <c r="AM13" s="13"/>
-    </row>
-    <row r="14" spans="1:39" x14ac:dyDescent="0.4">
+      <c r="AN13" s="13"/>
+    </row>
+    <row r="14" spans="1:40" x14ac:dyDescent="0.4">
       <c r="A14" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B14" s="6"/>
+      <c r="B14" s="4"/>
       <c r="C14" s="6"/>
       <c r="D14" s="6"/>
-      <c r="E14" s="17"/>
-      <c r="F14" s="6"/>
+      <c r="E14" s="6"/>
+      <c r="F14" s="17"/>
       <c r="G14" s="6"/>
-      <c r="H14" s="25" t="s">
+      <c r="H14" s="6"/>
+      <c r="I14" s="31" t="s">
         <v>20</v>
       </c>
-      <c r="I14" s="26"/>
       <c r="J14" s="26"/>
       <c r="K14" s="26"/>
       <c r="L14" s="26"/>
       <c r="M14" s="26"/>
-      <c r="N14" s="25" t="s">
+      <c r="N14" s="26"/>
+      <c r="O14" s="31" t="s">
         <v>22</v>
       </c>
-      <c r="O14" s="26"/>
       <c r="P14" s="26"/>
       <c r="Q14" s="26"/>
       <c r="R14" s="26"/>
       <c r="S14" s="26"/>
-      <c r="T14" s="26" t="s">
+      <c r="T14" s="26"/>
+      <c r="U14" s="26" t="s">
         <v>21</v>
       </c>
-      <c r="U14" s="26"/>
       <c r="V14" s="26"/>
       <c r="W14" s="26"/>
       <c r="X14" s="26"/>
@@ -1243,122 +1265,130 @@
       <c r="Z14" s="26"/>
       <c r="AA14" s="26"/>
       <c r="AB14" s="26"/>
-    </row>
-    <row r="15" spans="1:39" x14ac:dyDescent="0.4">
+      <c r="AC14" s="26"/>
+    </row>
+    <row r="15" spans="1:40" x14ac:dyDescent="0.4">
       <c r="A15" s="22" t="s">
         <v>34</v>
       </c>
-      <c r="B15" s="6"/>
+      <c r="B15" s="22"/>
       <c r="C15" s="6"/>
       <c r="D15" s="6"/>
-      <c r="AK15" s="13"/>
+      <c r="E15" s="6"/>
       <c r="AL15" s="13"/>
       <c r="AM15" s="13"/>
-    </row>
-    <row r="16" spans="1:39" x14ac:dyDescent="0.4">
+      <c r="AN15" s="13"/>
+    </row>
+    <row r="16" spans="1:40" x14ac:dyDescent="0.4">
       <c r="A16" s="19" t="s">
         <v>24</v>
       </c>
-      <c r="B16" s="6"/>
+      <c r="B16" s="19"/>
       <c r="C16" s="6"/>
       <c r="D16" s="6"/>
-    </row>
-    <row r="17" spans="1:39" x14ac:dyDescent="0.4">
+      <c r="E16" s="6"/>
+    </row>
+    <row r="17" spans="1:40" x14ac:dyDescent="0.4">
       <c r="A17" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="B17" s="24">
+      <c r="B17" s="4"/>
+      <c r="C17" s="32">
         <f>55/15</f>
         <v>3.6666666666666665</v>
       </c>
-      <c r="C17" s="24"/>
-      <c r="D17" s="24"/>
-      <c r="E17" s="3" t="s">
+      <c r="D17" s="32"/>
+      <c r="E17" s="32"/>
+      <c r="F17" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="AK17" s="13"/>
       <c r="AL17" s="13"/>
       <c r="AM17" s="13"/>
-    </row>
-    <row r="18" spans="1:39" x14ac:dyDescent="0.4">
+      <c r="AN17" s="13"/>
+    </row>
+    <row r="18" spans="1:40" x14ac:dyDescent="0.4">
       <c r="A18" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="B18" s="24">
+      <c r="B18" s="4"/>
+      <c r="C18" s="32">
         <f>65/15</f>
         <v>4.333333333333333</v>
       </c>
-      <c r="C18" s="24"/>
-      <c r="D18" s="24"/>
-      <c r="E18" s="3" t="s">
+      <c r="D18" s="32"/>
+      <c r="E18" s="32"/>
+      <c r="F18" s="3" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="19" spans="1:39" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:40" x14ac:dyDescent="0.4">
       <c r="A19" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B19" s="24">
+      <c r="B19" s="4"/>
+      <c r="C19" s="32">
         <f>75/15</f>
         <v>5</v>
       </c>
-      <c r="C19" s="24"/>
-      <c r="D19" s="24"/>
-      <c r="N19" s="15"/>
+      <c r="D19" s="32"/>
+      <c r="E19" s="32"/>
       <c r="O19" s="15"/>
       <c r="P19" s="15"/>
       <c r="Q19" s="15"/>
-    </row>
-    <row r="20" spans="1:39" x14ac:dyDescent="0.4">
+      <c r="R19" s="15"/>
+    </row>
+    <row r="20" spans="1:40" x14ac:dyDescent="0.4">
       <c r="A20" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="B20" s="24">
+      <c r="B20" s="4"/>
+      <c r="C20" s="32">
         <f>85/15</f>
         <v>5.666666666666667</v>
       </c>
-      <c r="C20" s="24"/>
-      <c r="D20" s="24"/>
-      <c r="N20" s="15"/>
+      <c r="D20" s="32"/>
+      <c r="E20" s="32"/>
       <c r="O20" s="15"/>
       <c r="P20" s="15"/>
       <c r="Q20" s="15"/>
-    </row>
-    <row r="21" spans="1:39" x14ac:dyDescent="0.4">
+      <c r="R20" s="15"/>
+    </row>
+    <row r="21" spans="1:40" x14ac:dyDescent="0.4">
       <c r="A21" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="B21" s="24">
+      <c r="B21" s="4"/>
+      <c r="C21" s="32">
         <f>95/15</f>
         <v>6.333333333333333</v>
       </c>
-      <c r="C21" s="24"/>
-      <c r="D21" s="24"/>
-      <c r="N21" s="15"/>
+      <c r="D21" s="32"/>
+      <c r="E21" s="32"/>
       <c r="O21" s="15"/>
       <c r="P21" s="15"/>
       <c r="Q21" s="15"/>
-    </row>
-    <row r="22" spans="1:39" x14ac:dyDescent="0.4">
+      <c r="R21" s="15"/>
+    </row>
+    <row r="22" spans="1:40" x14ac:dyDescent="0.4">
       <c r="A22" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B22" s="24">
+      <c r="B22" s="4"/>
+      <c r="C22" s="32">
         <f>105/15</f>
         <v>7</v>
       </c>
-      <c r="C22" s="24"/>
-      <c r="D22" s="24"/>
-      <c r="I22" s="6"/>
+      <c r="D22" s="32"/>
+      <c r="E22" s="32"/>
       <c r="J22" s="6"/>
       <c r="K22" s="6"/>
       <c r="L22" s="6"/>
       <c r="M22" s="6"/>
-      <c r="N22" s="15"/>
-      <c r="O22" s="16"/>
+      <c r="N22" s="6"/>
+      <c r="O22" s="15"/>
       <c r="P22" s="16"/>
       <c r="Q22" s="16"/>
-      <c r="R22" s="6"/>
+      <c r="R22" s="16"/>
       <c r="S22" s="6"/>
       <c r="T22" s="6"/>
       <c r="U22" s="6"/>
@@ -1367,21 +1397,22 @@
       <c r="X22" s="6"/>
       <c r="Y22" s="6"/>
       <c r="Z22" s="6"/>
-    </row>
-    <row r="23" spans="1:39" x14ac:dyDescent="0.4">
+      <c r="AA22" s="6"/>
+    </row>
+    <row r="23" spans="1:40" x14ac:dyDescent="0.4">
       <c r="A23" s="22" t="s">
         <v>35</v>
       </c>
-      <c r="I23" s="6"/>
+      <c r="B23" s="22"/>
       <c r="J23" s="6"/>
       <c r="K23" s="6"/>
       <c r="L23" s="6"/>
       <c r="M23" s="6"/>
-      <c r="N23" s="15"/>
-      <c r="O23" s="16"/>
+      <c r="N23" s="6"/>
+      <c r="O23" s="15"/>
       <c r="P23" s="16"/>
       <c r="Q23" s="16"/>
-      <c r="R23" s="6"/>
+      <c r="R23" s="16"/>
       <c r="S23" s="6"/>
       <c r="T23" s="6"/>
       <c r="U23" s="6"/>
@@ -1390,115 +1421,122 @@
       <c r="X23" s="6"/>
       <c r="Y23" s="6"/>
       <c r="Z23" s="6"/>
-    </row>
-    <row r="24" spans="1:39" x14ac:dyDescent="0.4">
+      <c r="AA23" s="6"/>
+    </row>
+    <row r="24" spans="1:40" x14ac:dyDescent="0.4">
       <c r="A24" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="B24" s="3" t="s">
+      <c r="B24" s="1"/>
+      <c r="C24" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="N24" s="15"/>
       <c r="O24" s="15"/>
       <c r="P24" s="15"/>
       <c r="Q24" s="15"/>
-    </row>
-    <row r="25" spans="1:39" x14ac:dyDescent="0.4">
+      <c r="R24" s="15"/>
+    </row>
+    <row r="25" spans="1:40" x14ac:dyDescent="0.4">
       <c r="A25" s="20" t="s">
         <v>37</v>
       </c>
-      <c r="B25" s="3" t="s">
+      <c r="B25" s="20"/>
+      <c r="C25" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="N25" s="15"/>
       <c r="O25" s="15"/>
       <c r="P25" s="15"/>
       <c r="Q25" s="15"/>
-    </row>
-    <row r="26" spans="1:39" x14ac:dyDescent="0.4">
+      <c r="R25" s="15"/>
+    </row>
+    <row r="26" spans="1:40" x14ac:dyDescent="0.4">
       <c r="A26" s="20" t="s">
         <v>38</v>
       </c>
-      <c r="B26" s="3" t="s">
+      <c r="B26" s="20"/>
+      <c r="C26" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="N26" s="15"/>
       <c r="O26" s="15"/>
       <c r="P26" s="15"/>
       <c r="Q26" s="15"/>
-    </row>
-    <row r="27" spans="1:39" x14ac:dyDescent="0.4">
+      <c r="R26" s="15"/>
+    </row>
+    <row r="27" spans="1:40" x14ac:dyDescent="0.4">
       <c r="A27" s="20" t="s">
         <v>39</v>
       </c>
-      <c r="B27" s="3" t="s">
+      <c r="B27" s="20"/>
+      <c r="C27" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="N27" s="15"/>
       <c r="O27" s="15"/>
       <c r="P27" s="15"/>
       <c r="Q27" s="15"/>
-    </row>
-    <row r="28" spans="1:39" x14ac:dyDescent="0.4">
+      <c r="R27" s="15"/>
+    </row>
+    <row r="28" spans="1:40" x14ac:dyDescent="0.4">
       <c r="A28" s="20"/>
-    </row>
-    <row r="29" spans="1:39" x14ac:dyDescent="0.4">
+      <c r="B28" s="20"/>
+    </row>
+    <row r="29" spans="1:40" x14ac:dyDescent="0.4">
       <c r="A29" s="20"/>
+      <c r="B29" s="20"/>
     </row>
   </sheetData>
   <mergeCells count="52">
-    <mergeCell ref="B7:D7"/>
-    <mergeCell ref="B5:D5"/>
-    <mergeCell ref="AC3:AH3"/>
-    <mergeCell ref="B6:D6"/>
-    <mergeCell ref="B3:D3"/>
-    <mergeCell ref="E3:G3"/>
-    <mergeCell ref="H3:K3"/>
-    <mergeCell ref="L3:Q3"/>
-    <mergeCell ref="R3:V3"/>
-    <mergeCell ref="W3:AB3"/>
-    <mergeCell ref="H7:K7"/>
-    <mergeCell ref="H6:K6"/>
-    <mergeCell ref="H5:K5"/>
-    <mergeCell ref="E7:G7"/>
-    <mergeCell ref="E6:G6"/>
-    <mergeCell ref="E5:G5"/>
-    <mergeCell ref="T14:AB14"/>
-    <mergeCell ref="W5:AB5"/>
-    <mergeCell ref="R7:V7"/>
-    <mergeCell ref="R6:V6"/>
-    <mergeCell ref="N11:S11"/>
-    <mergeCell ref="N12:S12"/>
-    <mergeCell ref="N13:S13"/>
-    <mergeCell ref="N14:S14"/>
-    <mergeCell ref="R5:V5"/>
-    <mergeCell ref="L7:Q7"/>
-    <mergeCell ref="L6:Q6"/>
-    <mergeCell ref="L5:Q5"/>
-    <mergeCell ref="T10:AB10"/>
-    <mergeCell ref="T11:AB11"/>
-    <mergeCell ref="T12:AB12"/>
-    <mergeCell ref="W6:AB6"/>
-    <mergeCell ref="T13:AB13"/>
-    <mergeCell ref="AC7:AH7"/>
-    <mergeCell ref="AC6:AH6"/>
-    <mergeCell ref="AC5:AH5"/>
-    <mergeCell ref="W7:AB7"/>
-    <mergeCell ref="T9:AB9"/>
-    <mergeCell ref="N9:S9"/>
-    <mergeCell ref="N10:S10"/>
-    <mergeCell ref="B21:D21"/>
-    <mergeCell ref="B17:D17"/>
-    <mergeCell ref="B18:D18"/>
-    <mergeCell ref="B19:D19"/>
-    <mergeCell ref="B20:D20"/>
-    <mergeCell ref="B22:D22"/>
-    <mergeCell ref="H9:M9"/>
-    <mergeCell ref="H10:M10"/>
-    <mergeCell ref="H11:M11"/>
-    <mergeCell ref="H12:M12"/>
-    <mergeCell ref="H13:M13"/>
-    <mergeCell ref="H14:M14"/>
+    <mergeCell ref="C22:E22"/>
+    <mergeCell ref="I9:N9"/>
+    <mergeCell ref="I10:N10"/>
+    <mergeCell ref="I11:N11"/>
+    <mergeCell ref="I12:N12"/>
+    <mergeCell ref="I13:N13"/>
+    <mergeCell ref="I14:N14"/>
+    <mergeCell ref="O9:T9"/>
+    <mergeCell ref="O10:T10"/>
+    <mergeCell ref="C21:E21"/>
+    <mergeCell ref="C17:E17"/>
+    <mergeCell ref="C18:E18"/>
+    <mergeCell ref="C19:E19"/>
+    <mergeCell ref="C20:E20"/>
+    <mergeCell ref="U13:AC13"/>
+    <mergeCell ref="AD7:AI7"/>
+    <mergeCell ref="AD6:AI6"/>
+    <mergeCell ref="AD5:AI5"/>
+    <mergeCell ref="X7:AC7"/>
+    <mergeCell ref="U9:AC9"/>
+    <mergeCell ref="U14:AC14"/>
+    <mergeCell ref="X5:AC5"/>
+    <mergeCell ref="S7:W7"/>
+    <mergeCell ref="S6:W6"/>
+    <mergeCell ref="O11:T11"/>
+    <mergeCell ref="O12:T12"/>
+    <mergeCell ref="O13:T13"/>
+    <mergeCell ref="O14:T14"/>
+    <mergeCell ref="S5:W5"/>
+    <mergeCell ref="M7:R7"/>
+    <mergeCell ref="M6:R6"/>
+    <mergeCell ref="M5:R5"/>
+    <mergeCell ref="U10:AC10"/>
+    <mergeCell ref="U11:AC11"/>
+    <mergeCell ref="U12:AC12"/>
+    <mergeCell ref="X6:AC6"/>
+    <mergeCell ref="C7:E7"/>
+    <mergeCell ref="C5:E5"/>
+    <mergeCell ref="AD3:AI3"/>
+    <mergeCell ref="C6:E6"/>
+    <mergeCell ref="C3:E3"/>
+    <mergeCell ref="F3:H3"/>
+    <mergeCell ref="I3:L3"/>
+    <mergeCell ref="M3:R3"/>
+    <mergeCell ref="S3:W3"/>
+    <mergeCell ref="X3:AC3"/>
+    <mergeCell ref="I7:L7"/>
+    <mergeCell ref="I6:L6"/>
+    <mergeCell ref="I5:L5"/>
+    <mergeCell ref="F7:H7"/>
+    <mergeCell ref="F6:H6"/>
+    <mergeCell ref="F5:H5"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="A1" r:id="rId1" xr:uid="{262308BA-9AEC-44C1-B6C0-92E820B5EA69}"/>

</xml_diff>

<commit_message>
Rename and update the recommendations to include skill levels
</commit_message>
<xml_diff>
--- a/data/research.xlsx
+++ b/data/research.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ninal\Desktop\projects\NinasProject\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3A8F283-A286-4E3C-8185-A2373BCFE143}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{453C454B-18B0-4133-92D4-0CC5AACD37CC}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="21585" windowHeight="8820" xr2:uid="{9C4ED264-3AF9-4DAD-A95C-E7848EE8F76F}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="48">
   <si>
     <t>&gt; 95</t>
   </si>
@@ -160,6 +160,15 @@
   </si>
   <si>
     <t>https://www.windcraftsurf.com/en/blog/beginners-guide-to-windsurfing</t>
+  </si>
+  <si>
+    <t>Wind Speed for Windsurfing: Knots to Plane (by Kit) | WindUp</t>
+  </si>
+  <si>
+    <t>If gusts are more than 8 knots above average, they are considered too strong (general rule).</t>
+  </si>
+  <si>
+    <t>If sail size is recommended for up to 12 knots and gusts are 20+ knots, they are too strong.</t>
   </si>
 </sst>
 </file>
@@ -169,7 +178,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -197,6 +206,38 @@
       <u/>
       <sz val="10"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <u/>
+      <sz val="10"/>
+      <color theme="0" tint="-0.34998626667073579"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="0" tint="-0.34998626667073579"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <u/>
+      <sz val="10"/>
+      <color theme="9" tint="0.79998168889431442"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="9" tint="0.79998168889431442"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -259,7 +300,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -268,9 +309,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -295,11 +333,7 @@
     <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -312,6 +346,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -329,20 +366,41 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -659,7 +717,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3B9AD222-34BA-409C-82CD-7E525C4015EB}">
-  <dimension ref="A1:AN29"/>
+  <dimension ref="A1:AN31"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="13.15" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="15.19921875" style="3" customWidth="1"/>
@@ -668,72 +726,72 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:40" ht="14.25" x14ac:dyDescent="0.45">
-      <c r="A1" s="23" t="s">
+      <c r="A1" s="20" t="s">
         <v>44</v>
       </c>
-      <c r="B1" s="23"/>
+      <c r="B1" s="20"/>
     </row>
     <row r="2" spans="1:40" x14ac:dyDescent="0.4">
-      <c r="A2" s="21" t="s">
+      <c r="A2" s="18" t="s">
         <v>33</v>
       </c>
-      <c r="B2" s="21"/>
+      <c r="B2" s="18"/>
     </row>
     <row r="3" spans="1:40" x14ac:dyDescent="0.4">
       <c r="A3" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="24">
+      <c r="B3" s="21">
         <v>0</v>
       </c>
-      <c r="C3" s="26">
+      <c r="C3" s="24">
         <v>1</v>
       </c>
-      <c r="D3" s="26"/>
-      <c r="E3" s="26"/>
-      <c r="F3" s="26">
+      <c r="D3" s="24"/>
+      <c r="E3" s="24"/>
+      <c r="F3" s="24">
         <v>2</v>
       </c>
-      <c r="G3" s="26"/>
-      <c r="H3" s="26"/>
-      <c r="I3" s="26">
+      <c r="G3" s="24"/>
+      <c r="H3" s="24"/>
+      <c r="I3" s="24">
         <v>3</v>
       </c>
-      <c r="J3" s="26"/>
-      <c r="K3" s="26"/>
-      <c r="L3" s="26"/>
-      <c r="M3" s="26">
+      <c r="J3" s="24"/>
+      <c r="K3" s="24"/>
+      <c r="L3" s="24"/>
+      <c r="M3" s="24">
         <v>4</v>
       </c>
-      <c r="N3" s="26"/>
-      <c r="O3" s="26"/>
-      <c r="P3" s="26"/>
-      <c r="Q3" s="26"/>
-      <c r="R3" s="26"/>
-      <c r="S3" s="26">
+      <c r="N3" s="24"/>
+      <c r="O3" s="24"/>
+      <c r="P3" s="24"/>
+      <c r="Q3" s="24"/>
+      <c r="R3" s="24"/>
+      <c r="S3" s="24">
         <v>5</v>
       </c>
-      <c r="T3" s="26"/>
-      <c r="U3" s="26"/>
-      <c r="V3" s="26"/>
-      <c r="W3" s="26"/>
-      <c r="X3" s="26">
+      <c r="T3" s="24"/>
+      <c r="U3" s="24"/>
+      <c r="V3" s="24"/>
+      <c r="W3" s="24"/>
+      <c r="X3" s="24">
         <v>6</v>
       </c>
-      <c r="Y3" s="26"/>
-      <c r="Z3" s="26"/>
-      <c r="AA3" s="26"/>
-      <c r="AB3" s="26"/>
-      <c r="AC3" s="26"/>
-      <c r="AD3" s="26">
+      <c r="Y3" s="24"/>
+      <c r="Z3" s="24"/>
+      <c r="AA3" s="24"/>
+      <c r="AB3" s="24"/>
+      <c r="AC3" s="24"/>
+      <c r="AD3" s="24">
         <v>7</v>
       </c>
-      <c r="AE3" s="26"/>
-      <c r="AF3" s="26"/>
-      <c r="AG3" s="26"/>
-      <c r="AH3" s="26"/>
-      <c r="AI3" s="26"/>
-      <c r="AK3" s="8" t="s">
+      <c r="AE3" s="24"/>
+      <c r="AF3" s="24"/>
+      <c r="AG3" s="24"/>
+      <c r="AH3" s="24"/>
+      <c r="AI3" s="24"/>
+      <c r="AK3" s="7" t="s">
         <v>4</v>
       </c>
     </row>
@@ -741,7 +799,7 @@
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="24">
+      <c r="B4" s="21">
         <v>0</v>
       </c>
       <c r="C4" s="2">
@@ -843,585 +901,618 @@
       <c r="AI4" s="2">
         <v>33</v>
       </c>
-      <c r="AK4" s="9" t="s">
+      <c r="AK4" s="8" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="5" spans="1:40" x14ac:dyDescent="0.4">
-      <c r="A5" s="7" t="s">
+      <c r="A5" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B5" s="35"/>
-      <c r="C5" s="25"/>
-      <c r="D5" s="25"/>
-      <c r="E5" s="25"/>
-      <c r="F5" s="27"/>
-      <c r="G5" s="27"/>
-      <c r="H5" s="27"/>
-      <c r="I5" s="28"/>
-      <c r="J5" s="28"/>
-      <c r="K5" s="28"/>
-      <c r="L5" s="28"/>
-      <c r="M5" s="30"/>
-      <c r="N5" s="30"/>
-      <c r="O5" s="30"/>
-      <c r="P5" s="30"/>
-      <c r="Q5" s="30"/>
-      <c r="R5" s="30"/>
-      <c r="S5" s="29"/>
-      <c r="T5" s="29"/>
-      <c r="U5" s="29"/>
-      <c r="V5" s="29"/>
-      <c r="W5" s="29"/>
-      <c r="X5" s="29"/>
-      <c r="Y5" s="29"/>
-      <c r="Z5" s="29"/>
-      <c r="AA5" s="29"/>
-      <c r="AB5" s="29"/>
-      <c r="AC5" s="29"/>
-      <c r="AD5" s="29"/>
-      <c r="AE5" s="29"/>
-      <c r="AF5" s="29"/>
-      <c r="AG5" s="29"/>
-      <c r="AH5" s="29"/>
-      <c r="AI5" s="29"/>
-      <c r="AK5" s="10" t="s">
+      <c r="B5" s="22"/>
+      <c r="C5" s="23"/>
+      <c r="D5" s="23"/>
+      <c r="E5" s="23"/>
+      <c r="F5" s="25"/>
+      <c r="G5" s="25"/>
+      <c r="H5" s="25"/>
+      <c r="I5" s="26"/>
+      <c r="J5" s="26"/>
+      <c r="K5" s="26"/>
+      <c r="L5" s="26"/>
+      <c r="M5" s="28"/>
+      <c r="N5" s="28"/>
+      <c r="O5" s="28"/>
+      <c r="P5" s="28"/>
+      <c r="Q5" s="28"/>
+      <c r="R5" s="28"/>
+      <c r="S5" s="27"/>
+      <c r="T5" s="27"/>
+      <c r="U5" s="27"/>
+      <c r="V5" s="27"/>
+      <c r="W5" s="27"/>
+      <c r="X5" s="27"/>
+      <c r="Y5" s="27"/>
+      <c r="Z5" s="27"/>
+      <c r="AA5" s="27"/>
+      <c r="AB5" s="27"/>
+      <c r="AC5" s="27"/>
+      <c r="AD5" s="27"/>
+      <c r="AE5" s="27"/>
+      <c r="AF5" s="27"/>
+      <c r="AG5" s="27"/>
+      <c r="AH5" s="27"/>
+      <c r="AI5" s="27"/>
+      <c r="AK5" s="9" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="6" spans="1:40" x14ac:dyDescent="0.4">
-      <c r="A6" s="7" t="s">
+      <c r="A6" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="B6" s="35"/>
-      <c r="C6" s="25"/>
-      <c r="D6" s="25"/>
-      <c r="E6" s="25"/>
-      <c r="F6" s="25"/>
-      <c r="G6" s="25"/>
-      <c r="H6" s="25"/>
-      <c r="I6" s="27"/>
-      <c r="J6" s="27"/>
-      <c r="K6" s="27"/>
-      <c r="L6" s="27"/>
-      <c r="M6" s="28"/>
-      <c r="N6" s="28"/>
-      <c r="O6" s="28"/>
-      <c r="P6" s="28"/>
-      <c r="Q6" s="28"/>
-      <c r="R6" s="28"/>
-      <c r="S6" s="30"/>
-      <c r="T6" s="30"/>
-      <c r="U6" s="30"/>
-      <c r="V6" s="30"/>
-      <c r="W6" s="30"/>
-      <c r="X6" s="29"/>
-      <c r="Y6" s="29"/>
-      <c r="Z6" s="29"/>
-      <c r="AA6" s="29"/>
-      <c r="AB6" s="29"/>
-      <c r="AC6" s="29"/>
-      <c r="AD6" s="29"/>
-      <c r="AE6" s="29"/>
-      <c r="AF6" s="29"/>
-      <c r="AG6" s="29"/>
-      <c r="AH6" s="29"/>
-      <c r="AI6" s="29"/>
-      <c r="AJ6" s="5"/>
-      <c r="AK6" s="11" t="s">
+      <c r="B6" s="22"/>
+      <c r="C6" s="23"/>
+      <c r="D6" s="23"/>
+      <c r="E6" s="23"/>
+      <c r="F6" s="23"/>
+      <c r="G6" s="23"/>
+      <c r="H6" s="23"/>
+      <c r="I6" s="25"/>
+      <c r="J6" s="25"/>
+      <c r="K6" s="25"/>
+      <c r="L6" s="25"/>
+      <c r="M6" s="26"/>
+      <c r="N6" s="26"/>
+      <c r="O6" s="26"/>
+      <c r="P6" s="26"/>
+      <c r="Q6" s="26"/>
+      <c r="R6" s="26"/>
+      <c r="S6" s="28"/>
+      <c r="T6" s="28"/>
+      <c r="U6" s="28"/>
+      <c r="V6" s="28"/>
+      <c r="W6" s="28"/>
+      <c r="X6" s="27"/>
+      <c r="Y6" s="27"/>
+      <c r="Z6" s="27"/>
+      <c r="AA6" s="27"/>
+      <c r="AB6" s="27"/>
+      <c r="AC6" s="27"/>
+      <c r="AD6" s="27"/>
+      <c r="AE6" s="27"/>
+      <c r="AF6" s="27"/>
+      <c r="AG6" s="27"/>
+      <c r="AH6" s="27"/>
+      <c r="AI6" s="27"/>
+      <c r="AJ6" s="4"/>
+      <c r="AK6" s="10" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="7" spans="1:40" x14ac:dyDescent="0.4">
-      <c r="A7" s="7" t="s">
+      <c r="A7" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="B7" s="35"/>
-      <c r="C7" s="25"/>
-      <c r="D7" s="25"/>
-      <c r="E7" s="25"/>
-      <c r="F7" s="25"/>
-      <c r="G7" s="25"/>
-      <c r="H7" s="25"/>
-      <c r="I7" s="27"/>
-      <c r="J7" s="27"/>
-      <c r="K7" s="27"/>
-      <c r="L7" s="27"/>
-      <c r="M7" s="27"/>
-      <c r="N7" s="27"/>
-      <c r="O7" s="27"/>
-      <c r="P7" s="27"/>
-      <c r="Q7" s="27"/>
-      <c r="R7" s="27"/>
-      <c r="S7" s="28"/>
-      <c r="T7" s="28"/>
-      <c r="U7" s="28"/>
-      <c r="V7" s="28"/>
-      <c r="W7" s="28"/>
-      <c r="X7" s="30"/>
-      <c r="Y7" s="30"/>
-      <c r="Z7" s="30"/>
-      <c r="AA7" s="30"/>
-      <c r="AB7" s="30"/>
-      <c r="AC7" s="30"/>
-      <c r="AD7" s="29"/>
-      <c r="AE7" s="29"/>
-      <c r="AF7" s="29"/>
-      <c r="AG7" s="29"/>
-      <c r="AH7" s="29"/>
-      <c r="AI7" s="29"/>
-      <c r="AK7" s="12" t="s">
+      <c r="B7" s="22"/>
+      <c r="C7" s="23"/>
+      <c r="D7" s="23"/>
+      <c r="E7" s="23"/>
+      <c r="F7" s="23"/>
+      <c r="G7" s="23"/>
+      <c r="H7" s="23"/>
+      <c r="I7" s="25"/>
+      <c r="J7" s="25"/>
+      <c r="K7" s="25"/>
+      <c r="L7" s="25"/>
+      <c r="M7" s="25"/>
+      <c r="N7" s="25"/>
+      <c r="O7" s="25"/>
+      <c r="P7" s="25"/>
+      <c r="Q7" s="25"/>
+      <c r="R7" s="25"/>
+      <c r="S7" s="26"/>
+      <c r="T7" s="26"/>
+      <c r="U7" s="26"/>
+      <c r="V7" s="26"/>
+      <c r="W7" s="26"/>
+      <c r="X7" s="28"/>
+      <c r="Y7" s="28"/>
+      <c r="Z7" s="28"/>
+      <c r="AA7" s="28"/>
+      <c r="AB7" s="28"/>
+      <c r="AC7" s="28"/>
+      <c r="AD7" s="27"/>
+      <c r="AE7" s="27"/>
+      <c r="AF7" s="27"/>
+      <c r="AG7" s="27"/>
+      <c r="AH7" s="27"/>
+      <c r="AI7" s="27"/>
+      <c r="AK7" s="11" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="8" spans="1:40" x14ac:dyDescent="0.4">
-      <c r="A8" s="22" t="s">
+      <c r="A8" s="29" t="s">
         <v>32</v>
       </c>
-      <c r="B8" s="22"/>
-      <c r="C8" s="6"/>
-      <c r="D8" s="6"/>
-      <c r="E8" s="6"/>
+      <c r="B8" s="29"/>
+      <c r="C8" s="30"/>
+      <c r="D8" s="30"/>
+      <c r="E8" s="30"/>
+      <c r="F8" s="31"/>
+      <c r="G8" s="31"/>
+      <c r="H8" s="31"/>
+      <c r="I8" s="31"/>
+      <c r="J8" s="31"/>
+      <c r="K8" s="31"/>
+      <c r="L8" s="31"/>
+      <c r="M8" s="31"/>
+      <c r="N8" s="31"/>
+      <c r="O8" s="31"/>
+      <c r="P8" s="31"/>
+      <c r="Q8" s="31"/>
+      <c r="R8" s="31"/>
+      <c r="S8" s="31"/>
+      <c r="T8" s="31"/>
+      <c r="U8" s="31"/>
+      <c r="V8" s="31"/>
+      <c r="W8" s="31"/>
+      <c r="X8" s="31"/>
+      <c r="Y8" s="31"/>
+      <c r="Z8" s="31"/>
+      <c r="AA8" s="31"/>
+      <c r="AB8" s="31"/>
+      <c r="AC8" s="31"/>
+      <c r="AD8" s="31"/>
     </row>
     <row r="9" spans="1:40" x14ac:dyDescent="0.4">
-      <c r="A9" s="4" t="s">
+      <c r="A9" s="32" t="s">
         <v>1</v>
       </c>
-      <c r="B9" s="4"/>
-      <c r="C9" s="6"/>
-      <c r="D9" s="6"/>
-      <c r="E9" s="6"/>
-      <c r="G9" s="6"/>
-      <c r="H9" s="6"/>
-      <c r="I9" s="31" t="s">
+      <c r="B9" s="32"/>
+      <c r="C9" s="30"/>
+      <c r="D9" s="30"/>
+      <c r="E9" s="30"/>
+      <c r="F9" s="31"/>
+      <c r="G9" s="30"/>
+      <c r="H9" s="30"/>
+      <c r="I9" s="33" t="s">
         <v>18</v>
       </c>
-      <c r="J9" s="26"/>
-      <c r="K9" s="26"/>
-      <c r="L9" s="26"/>
-      <c r="M9" s="26"/>
-      <c r="N9" s="26"/>
-      <c r="O9" s="31" t="s">
+      <c r="J9" s="34"/>
+      <c r="K9" s="34"/>
+      <c r="L9" s="34"/>
+      <c r="M9" s="34"/>
+      <c r="N9" s="34"/>
+      <c r="O9" s="33" t="s">
         <v>12</v>
       </c>
-      <c r="P9" s="26"/>
-      <c r="Q9" s="26"/>
-      <c r="R9" s="26"/>
-      <c r="S9" s="26"/>
-      <c r="T9" s="26"/>
-      <c r="U9" s="31" t="s">
+      <c r="P9" s="34"/>
+      <c r="Q9" s="34"/>
+      <c r="R9" s="34"/>
+      <c r="S9" s="34"/>
+      <c r="T9" s="34"/>
+      <c r="U9" s="33" t="s">
         <v>23</v>
       </c>
-      <c r="V9" s="26"/>
-      <c r="W9" s="26"/>
-      <c r="X9" s="26"/>
-      <c r="Y9" s="26"/>
-      <c r="Z9" s="26"/>
-      <c r="AA9" s="26"/>
-      <c r="AB9" s="26"/>
-      <c r="AC9" s="26"/>
-      <c r="AD9" s="14" t="s">
+      <c r="V9" s="34"/>
+      <c r="W9" s="34"/>
+      <c r="X9" s="34"/>
+      <c r="Y9" s="34"/>
+      <c r="Z9" s="34"/>
+      <c r="AA9" s="34"/>
+      <c r="AB9" s="34"/>
+      <c r="AC9" s="34"/>
+      <c r="AD9" s="35" t="s">
         <v>26</v>
       </c>
-      <c r="AE9" s="14"/>
-      <c r="AF9" s="14"/>
-      <c r="AG9" s="14"/>
-      <c r="AH9" s="14"/>
-      <c r="AI9" s="14"/>
-      <c r="AK9" s="18"/>
+      <c r="AE9" s="13"/>
+      <c r="AF9" s="13"/>
+      <c r="AG9" s="13"/>
+      <c r="AH9" s="13"/>
+      <c r="AI9" s="13"/>
+      <c r="AK9" s="16"/>
     </row>
     <row r="10" spans="1:40" x14ac:dyDescent="0.4">
-      <c r="A10" s="4" t="s">
+      <c r="A10" s="32" t="s">
         <v>14</v>
       </c>
-      <c r="B10" s="4"/>
-      <c r="C10" s="6"/>
-      <c r="D10" s="6"/>
-      <c r="E10" s="6"/>
-      <c r="F10" s="17"/>
-      <c r="G10" s="6"/>
-      <c r="H10" s="6"/>
-      <c r="I10" s="31" t="s">
+      <c r="B10" s="32"/>
+      <c r="C10" s="30"/>
+      <c r="D10" s="30"/>
+      <c r="E10" s="30"/>
+      <c r="F10" s="36"/>
+      <c r="G10" s="30"/>
+      <c r="H10" s="30"/>
+      <c r="I10" s="33" t="s">
         <v>19</v>
       </c>
-      <c r="J10" s="26"/>
-      <c r="K10" s="26"/>
-      <c r="L10" s="26"/>
-      <c r="M10" s="26"/>
-      <c r="N10" s="26"/>
-      <c r="O10" s="31" t="s">
+      <c r="J10" s="34"/>
+      <c r="K10" s="34"/>
+      <c r="L10" s="34"/>
+      <c r="M10" s="34"/>
+      <c r="N10" s="34"/>
+      <c r="O10" s="33" t="s">
         <v>18</v>
       </c>
-      <c r="P10" s="26"/>
-      <c r="Q10" s="26"/>
-      <c r="R10" s="26"/>
-      <c r="S10" s="26"/>
-      <c r="T10" s="26"/>
-      <c r="U10" s="26" t="s">
+      <c r="P10" s="34"/>
+      <c r="Q10" s="34"/>
+      <c r="R10" s="34"/>
+      <c r="S10" s="34"/>
+      <c r="T10" s="34"/>
+      <c r="U10" s="34" t="s">
         <v>12</v>
       </c>
-      <c r="V10" s="26"/>
-      <c r="W10" s="26"/>
-      <c r="X10" s="26"/>
-      <c r="Y10" s="26"/>
-      <c r="Z10" s="26"/>
-      <c r="AA10" s="26"/>
-      <c r="AB10" s="26"/>
-      <c r="AC10" s="26"/>
-      <c r="AD10" s="14" t="s">
+      <c r="V10" s="34"/>
+      <c r="W10" s="34"/>
+      <c r="X10" s="34"/>
+      <c r="Y10" s="34"/>
+      <c r="Z10" s="34"/>
+      <c r="AA10" s="34"/>
+      <c r="AB10" s="34"/>
+      <c r="AC10" s="34"/>
+      <c r="AD10" s="35" t="s">
         <v>27</v>
       </c>
-      <c r="AE10" s="14"/>
-      <c r="AF10" s="14"/>
-      <c r="AG10" s="14"/>
-      <c r="AH10" s="14"/>
-      <c r="AI10" s="14"/>
-      <c r="AK10" s="15"/>
-      <c r="AL10" s="13"/>
-      <c r="AM10" s="13"/>
-      <c r="AN10" s="13"/>
+      <c r="AE10" s="13"/>
+      <c r="AF10" s="13"/>
+      <c r="AG10" s="13"/>
+      <c r="AH10" s="13"/>
+      <c r="AI10" s="13"/>
+      <c r="AK10" s="14"/>
+      <c r="AL10" s="12"/>
+      <c r="AM10" s="12"/>
+      <c r="AN10" s="12"/>
     </row>
     <row r="11" spans="1:40" x14ac:dyDescent="0.4">
-      <c r="A11" s="4" t="s">
+      <c r="A11" s="32" t="s">
         <v>15</v>
       </c>
-      <c r="B11" s="4"/>
-      <c r="C11" s="6"/>
-      <c r="D11" s="6"/>
-      <c r="E11" s="6"/>
-      <c r="F11" s="17"/>
-      <c r="G11" s="6"/>
-      <c r="H11" s="6"/>
-      <c r="I11" s="31" t="s">
+      <c r="B11" s="32"/>
+      <c r="C11" s="30"/>
+      <c r="D11" s="30"/>
+      <c r="E11" s="30"/>
+      <c r="F11" s="36"/>
+      <c r="G11" s="30"/>
+      <c r="H11" s="30"/>
+      <c r="I11" s="33" t="s">
         <v>13</v>
       </c>
-      <c r="J11" s="26"/>
-      <c r="K11" s="26"/>
-      <c r="L11" s="26"/>
-      <c r="M11" s="26"/>
-      <c r="N11" s="26"/>
-      <c r="O11" s="31" t="s">
+      <c r="J11" s="34"/>
+      <c r="K11" s="34"/>
+      <c r="L11" s="34"/>
+      <c r="M11" s="34"/>
+      <c r="N11" s="34"/>
+      <c r="O11" s="33" t="s">
         <v>19</v>
       </c>
-      <c r="P11" s="26"/>
-      <c r="Q11" s="26"/>
-      <c r="R11" s="26"/>
-      <c r="S11" s="26"/>
-      <c r="T11" s="26"/>
-      <c r="U11" s="26" t="s">
+      <c r="P11" s="34"/>
+      <c r="Q11" s="34"/>
+      <c r="R11" s="34"/>
+      <c r="S11" s="34"/>
+      <c r="T11" s="34"/>
+      <c r="U11" s="34" t="s">
         <v>18</v>
       </c>
-      <c r="V11" s="26"/>
-      <c r="W11" s="26"/>
-      <c r="X11" s="26"/>
-      <c r="Y11" s="26"/>
-      <c r="Z11" s="26"/>
-      <c r="AA11" s="26"/>
-      <c r="AB11" s="26"/>
-      <c r="AC11" s="26"/>
-      <c r="AD11" s="14" t="s">
+      <c r="V11" s="34"/>
+      <c r="W11" s="34"/>
+      <c r="X11" s="34"/>
+      <c r="Y11" s="34"/>
+      <c r="Z11" s="34"/>
+      <c r="AA11" s="34"/>
+      <c r="AB11" s="34"/>
+      <c r="AC11" s="34"/>
+      <c r="AD11" s="35" t="s">
         <v>28</v>
       </c>
-      <c r="AE11" s="14"/>
-      <c r="AF11" s="14"/>
-      <c r="AG11" s="14"/>
-      <c r="AH11" s="14"/>
-      <c r="AI11" s="14"/>
-      <c r="AK11" s="15"/>
+      <c r="AE11" s="13"/>
+      <c r="AF11" s="13"/>
+      <c r="AG11" s="13"/>
+      <c r="AH11" s="13"/>
+      <c r="AI11" s="13"/>
+      <c r="AK11" s="14"/>
     </row>
     <row r="12" spans="1:40" x14ac:dyDescent="0.4">
-      <c r="A12" s="4" t="s">
+      <c r="A12" s="32" t="s">
         <v>16</v>
       </c>
-      <c r="B12" s="4"/>
-      <c r="C12" s="6"/>
-      <c r="D12" s="6"/>
-      <c r="E12" s="6"/>
-      <c r="F12" s="17"/>
-      <c r="G12" s="6"/>
-      <c r="H12" s="6"/>
-      <c r="I12" s="33" t="s">
+      <c r="B12" s="32"/>
+      <c r="C12" s="30"/>
+      <c r="D12" s="30"/>
+      <c r="E12" s="30"/>
+      <c r="F12" s="36"/>
+      <c r="G12" s="30"/>
+      <c r="H12" s="30"/>
+      <c r="I12" s="37" t="s">
         <v>21</v>
       </c>
-      <c r="J12" s="34"/>
-      <c r="K12" s="34"/>
-      <c r="L12" s="34"/>
-      <c r="M12" s="34"/>
-      <c r="N12" s="34"/>
-      <c r="O12" s="31" t="s">
+      <c r="J12" s="38"/>
+      <c r="K12" s="38"/>
+      <c r="L12" s="38"/>
+      <c r="M12" s="38"/>
+      <c r="N12" s="38"/>
+      <c r="O12" s="33" t="s">
         <v>13</v>
       </c>
-      <c r="P12" s="26"/>
-      <c r="Q12" s="26"/>
-      <c r="R12" s="26"/>
-      <c r="S12" s="26"/>
-      <c r="T12" s="26"/>
-      <c r="U12" s="26" t="s">
+      <c r="P12" s="34"/>
+      <c r="Q12" s="34"/>
+      <c r="R12" s="34"/>
+      <c r="S12" s="34"/>
+      <c r="T12" s="34"/>
+      <c r="U12" s="34" t="s">
         <v>19</v>
       </c>
-      <c r="V12" s="26"/>
-      <c r="W12" s="26"/>
-      <c r="X12" s="26"/>
-      <c r="Y12" s="26"/>
-      <c r="Z12" s="26"/>
-      <c r="AA12" s="26"/>
-      <c r="AB12" s="26"/>
-      <c r="AC12" s="26"/>
-      <c r="AD12" s="14" t="s">
+      <c r="V12" s="34"/>
+      <c r="W12" s="34"/>
+      <c r="X12" s="34"/>
+      <c r="Y12" s="34"/>
+      <c r="Z12" s="34"/>
+      <c r="AA12" s="34"/>
+      <c r="AB12" s="34"/>
+      <c r="AC12" s="34"/>
+      <c r="AD12" s="35" t="s">
         <v>29</v>
       </c>
-      <c r="AE12" s="14"/>
-      <c r="AF12" s="14"/>
-      <c r="AG12" s="14"/>
-      <c r="AH12" s="14"/>
-      <c r="AI12" s="14"/>
-      <c r="AK12" s="15"/>
+      <c r="AE12" s="13"/>
+      <c r="AF12" s="13"/>
+      <c r="AG12" s="13"/>
+      <c r="AH12" s="13"/>
+      <c r="AI12" s="13"/>
+      <c r="AK12" s="14"/>
     </row>
     <row r="13" spans="1:40" x14ac:dyDescent="0.4">
-      <c r="A13" s="4" t="s">
+      <c r="A13" s="32" t="s">
         <v>17</v>
       </c>
-      <c r="B13" s="4"/>
-      <c r="C13" s="6"/>
-      <c r="D13" s="6"/>
-      <c r="E13" s="6"/>
-      <c r="F13" s="17"/>
-      <c r="G13" s="6"/>
-      <c r="H13" s="6"/>
-      <c r="I13" s="33" t="s">
+      <c r="B13" s="32"/>
+      <c r="C13" s="30"/>
+      <c r="D13" s="30"/>
+      <c r="E13" s="30"/>
+      <c r="F13" s="36"/>
+      <c r="G13" s="30"/>
+      <c r="H13" s="30"/>
+      <c r="I13" s="37" t="s">
         <v>22</v>
       </c>
-      <c r="J13" s="34"/>
-      <c r="K13" s="34"/>
-      <c r="L13" s="34"/>
-      <c r="M13" s="34"/>
-      <c r="N13" s="34"/>
-      <c r="O13" s="31" t="s">
+      <c r="J13" s="38"/>
+      <c r="K13" s="38"/>
+      <c r="L13" s="38"/>
+      <c r="M13" s="38"/>
+      <c r="N13" s="38"/>
+      <c r="O13" s="33" t="s">
         <v>21</v>
       </c>
-      <c r="P13" s="26"/>
-      <c r="Q13" s="26"/>
-      <c r="R13" s="26"/>
-      <c r="S13" s="26"/>
-      <c r="T13" s="26"/>
-      <c r="U13" s="26" t="s">
+      <c r="P13" s="34"/>
+      <c r="Q13" s="34"/>
+      <c r="R13" s="34"/>
+      <c r="S13" s="34"/>
+      <c r="T13" s="34"/>
+      <c r="U13" s="34" t="s">
         <v>13</v>
       </c>
-      <c r="V13" s="26"/>
-      <c r="W13" s="26"/>
-      <c r="X13" s="26"/>
-      <c r="Y13" s="26"/>
-      <c r="Z13" s="26"/>
-      <c r="AA13" s="26"/>
-      <c r="AB13" s="26"/>
-      <c r="AC13" s="26"/>
-      <c r="AD13" s="14" t="s">
+      <c r="V13" s="34"/>
+      <c r="W13" s="34"/>
+      <c r="X13" s="34"/>
+      <c r="Y13" s="34"/>
+      <c r="Z13" s="34"/>
+      <c r="AA13" s="34"/>
+      <c r="AB13" s="34"/>
+      <c r="AC13" s="34"/>
+      <c r="AD13" s="35" t="s">
         <v>30</v>
       </c>
-      <c r="AE13" s="14"/>
-      <c r="AF13" s="14"/>
-      <c r="AG13" s="14"/>
-      <c r="AH13" s="14"/>
-      <c r="AI13" s="14"/>
-      <c r="AK13" s="15"/>
-      <c r="AL13" s="13"/>
-      <c r="AM13" s="13"/>
-      <c r="AN13" s="13"/>
+      <c r="AE13" s="13"/>
+      <c r="AF13" s="13"/>
+      <c r="AG13" s="13"/>
+      <c r="AH13" s="13"/>
+      <c r="AI13" s="13"/>
+      <c r="AK13" s="14"/>
+      <c r="AL13" s="12"/>
+      <c r="AM13" s="12"/>
+      <c r="AN13" s="12"/>
     </row>
     <row r="14" spans="1:40" x14ac:dyDescent="0.4">
-      <c r="A14" s="4" t="s">
+      <c r="A14" s="32" t="s">
         <v>0</v>
       </c>
-      <c r="B14" s="4"/>
-      <c r="C14" s="6"/>
-      <c r="D14" s="6"/>
-      <c r="E14" s="6"/>
-      <c r="F14" s="17"/>
-      <c r="G14" s="6"/>
-      <c r="H14" s="6"/>
-      <c r="I14" s="31" t="s">
+      <c r="B14" s="32"/>
+      <c r="C14" s="30"/>
+      <c r="D14" s="30"/>
+      <c r="E14" s="30"/>
+      <c r="F14" s="36"/>
+      <c r="G14" s="30"/>
+      <c r="H14" s="30"/>
+      <c r="I14" s="33" t="s">
         <v>20</v>
       </c>
-      <c r="J14" s="26"/>
-      <c r="K14" s="26"/>
-      <c r="L14" s="26"/>
-      <c r="M14" s="26"/>
-      <c r="N14" s="26"/>
-      <c r="O14" s="31" t="s">
+      <c r="J14" s="34"/>
+      <c r="K14" s="34"/>
+      <c r="L14" s="34"/>
+      <c r="M14" s="34"/>
+      <c r="N14" s="34"/>
+      <c r="O14" s="33" t="s">
         <v>22</v>
       </c>
-      <c r="P14" s="26"/>
-      <c r="Q14" s="26"/>
-      <c r="R14" s="26"/>
-      <c r="S14" s="26"/>
-      <c r="T14" s="26"/>
-      <c r="U14" s="26" t="s">
+      <c r="P14" s="34"/>
+      <c r="Q14" s="34"/>
+      <c r="R14" s="34"/>
+      <c r="S14" s="34"/>
+      <c r="T14" s="34"/>
+      <c r="U14" s="34" t="s">
         <v>21</v>
       </c>
-      <c r="V14" s="26"/>
-      <c r="W14" s="26"/>
-      <c r="X14" s="26"/>
-      <c r="Y14" s="26"/>
-      <c r="Z14" s="26"/>
-      <c r="AA14" s="26"/>
-      <c r="AB14" s="26"/>
-      <c r="AC14" s="26"/>
+      <c r="V14" s="34"/>
+      <c r="W14" s="34"/>
+      <c r="X14" s="34"/>
+      <c r="Y14" s="34"/>
+      <c r="Z14" s="34"/>
+      <c r="AA14" s="34"/>
+      <c r="AB14" s="34"/>
+      <c r="AC14" s="34"/>
+      <c r="AD14" s="31"/>
     </row>
     <row r="15" spans="1:40" x14ac:dyDescent="0.4">
-      <c r="A15" s="22" t="s">
+      <c r="A15" s="39" t="s">
         <v>34</v>
       </c>
-      <c r="B15" s="22"/>
-      <c r="C15" s="6"/>
-      <c r="D15" s="6"/>
-      <c r="E15" s="6"/>
-      <c r="AL15" s="13"/>
-      <c r="AM15" s="13"/>
-      <c r="AN15" s="13"/>
+      <c r="B15" s="39"/>
+      <c r="C15" s="40"/>
+      <c r="D15" s="40"/>
+      <c r="E15" s="40"/>
+      <c r="F15" s="41"/>
+      <c r="AL15" s="12"/>
+      <c r="AM15" s="12"/>
+      <c r="AN15" s="12"/>
     </row>
     <row r="16" spans="1:40" x14ac:dyDescent="0.4">
-      <c r="A16" s="19" t="s">
+      <c r="A16" s="42" t="s">
         <v>24</v>
       </c>
-      <c r="B16" s="19"/>
-      <c r="C16" s="6"/>
-      <c r="D16" s="6"/>
-      <c r="E16" s="6"/>
+      <c r="B16" s="42"/>
+      <c r="C16" s="40"/>
+      <c r="D16" s="40"/>
+      <c r="E16" s="40"/>
+      <c r="F16" s="41"/>
     </row>
     <row r="17" spans="1:40" x14ac:dyDescent="0.4">
-      <c r="A17" s="4" t="s">
+      <c r="A17" s="43" t="s">
         <v>1</v>
       </c>
-      <c r="B17" s="4"/>
-      <c r="C17" s="32">
+      <c r="B17" s="43"/>
+      <c r="C17" s="44">
         <f>55/15</f>
         <v>3.6666666666666665</v>
       </c>
-      <c r="D17" s="32"/>
-      <c r="E17" s="32"/>
-      <c r="F17" s="3" t="s">
+      <c r="D17" s="44"/>
+      <c r="E17" s="44"/>
+      <c r="F17" s="41" t="s">
         <v>25</v>
       </c>
-      <c r="AL17" s="13"/>
-      <c r="AM17" s="13"/>
-      <c r="AN17" s="13"/>
+      <c r="AL17" s="12"/>
+      <c r="AM17" s="12"/>
+      <c r="AN17" s="12"/>
     </row>
     <row r="18" spans="1:40" x14ac:dyDescent="0.4">
-      <c r="A18" s="4" t="s">
+      <c r="A18" s="43" t="s">
         <v>14</v>
       </c>
-      <c r="B18" s="4"/>
-      <c r="C18" s="32">
+      <c r="B18" s="43"/>
+      <c r="C18" s="44">
         <f>65/15</f>
         <v>4.333333333333333</v>
       </c>
-      <c r="D18" s="32"/>
-      <c r="E18" s="32"/>
-      <c r="F18" s="3" t="s">
+      <c r="D18" s="44"/>
+      <c r="E18" s="44"/>
+      <c r="F18" s="41" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="19" spans="1:40" x14ac:dyDescent="0.4">
-      <c r="A19" s="4" t="s">
+      <c r="A19" s="43" t="s">
         <v>15</v>
       </c>
-      <c r="B19" s="4"/>
-      <c r="C19" s="32">
+      <c r="B19" s="43"/>
+      <c r="C19" s="44">
         <f>75/15</f>
         <v>5</v>
       </c>
-      <c r="D19" s="32"/>
-      <c r="E19" s="32"/>
-      <c r="O19" s="15"/>
-      <c r="P19" s="15"/>
-      <c r="Q19" s="15"/>
-      <c r="R19" s="15"/>
+      <c r="D19" s="44"/>
+      <c r="E19" s="44"/>
+      <c r="F19" s="41"/>
+      <c r="O19" s="14"/>
+      <c r="P19" s="14"/>
+      <c r="Q19" s="14"/>
+      <c r="R19" s="14"/>
     </row>
     <row r="20" spans="1:40" x14ac:dyDescent="0.4">
-      <c r="A20" s="4" t="s">
+      <c r="A20" s="43" t="s">
         <v>16</v>
       </c>
-      <c r="B20" s="4"/>
-      <c r="C20" s="32">
+      <c r="B20" s="43"/>
+      <c r="C20" s="44">
         <f>85/15</f>
         <v>5.666666666666667</v>
       </c>
-      <c r="D20" s="32"/>
-      <c r="E20" s="32"/>
-      <c r="O20" s="15"/>
-      <c r="P20" s="15"/>
-      <c r="Q20" s="15"/>
-      <c r="R20" s="15"/>
+      <c r="D20" s="44"/>
+      <c r="E20" s="44"/>
+      <c r="F20" s="41"/>
+      <c r="O20" s="14"/>
+      <c r="P20" s="14"/>
+      <c r="Q20" s="14"/>
+      <c r="R20" s="14"/>
     </row>
     <row r="21" spans="1:40" x14ac:dyDescent="0.4">
-      <c r="A21" s="4" t="s">
+      <c r="A21" s="43" t="s">
         <v>17</v>
       </c>
-      <c r="B21" s="4"/>
-      <c r="C21" s="32">
+      <c r="B21" s="43"/>
+      <c r="C21" s="44">
         <f>95/15</f>
         <v>6.333333333333333</v>
       </c>
-      <c r="D21" s="32"/>
-      <c r="E21" s="32"/>
-      <c r="O21" s="15"/>
-      <c r="P21" s="15"/>
-      <c r="Q21" s="15"/>
-      <c r="R21" s="15"/>
+      <c r="D21" s="44"/>
+      <c r="E21" s="44"/>
+      <c r="F21" s="41"/>
+      <c r="O21" s="14"/>
+      <c r="P21" s="14"/>
+      <c r="Q21" s="14"/>
+      <c r="R21" s="14"/>
     </row>
     <row r="22" spans="1:40" x14ac:dyDescent="0.4">
-      <c r="A22" s="4" t="s">
+      <c r="A22" s="43" t="s">
         <v>0</v>
       </c>
-      <c r="B22" s="4"/>
-      <c r="C22" s="32">
+      <c r="B22" s="43"/>
+      <c r="C22" s="44">
         <f>105/15</f>
         <v>7</v>
       </c>
-      <c r="D22" s="32"/>
-      <c r="E22" s="32"/>
-      <c r="J22" s="6"/>
-      <c r="K22" s="6"/>
-      <c r="L22" s="6"/>
-      <c r="M22" s="6"/>
-      <c r="N22" s="6"/>
-      <c r="O22" s="15"/>
-      <c r="P22" s="16"/>
-      <c r="Q22" s="16"/>
-      <c r="R22" s="16"/>
-      <c r="S22" s="6"/>
-      <c r="T22" s="6"/>
-      <c r="U22" s="6"/>
-      <c r="V22" s="6"/>
-      <c r="W22" s="6"/>
-      <c r="X22" s="6"/>
-      <c r="Y22" s="6"/>
-      <c r="Z22" s="6"/>
-      <c r="AA22" s="6"/>
+      <c r="D22" s="44"/>
+      <c r="E22" s="44"/>
+      <c r="F22" s="41"/>
+      <c r="J22" s="5"/>
+      <c r="K22" s="5"/>
+      <c r="L22" s="5"/>
+      <c r="M22" s="5"/>
+      <c r="N22" s="5"/>
+      <c r="O22" s="14"/>
+      <c r="P22" s="15"/>
+      <c r="Q22" s="15"/>
+      <c r="R22" s="15"/>
+      <c r="S22" s="5"/>
+      <c r="T22" s="5"/>
+      <c r="U22" s="5"/>
+      <c r="V22" s="5"/>
+      <c r="W22" s="5"/>
+      <c r="X22" s="5"/>
+      <c r="Y22" s="5"/>
+      <c r="Z22" s="5"/>
+      <c r="AA22" s="5"/>
     </row>
     <row r="23" spans="1:40" x14ac:dyDescent="0.4">
-      <c r="A23" s="22" t="s">
+      <c r="A23" s="19" t="s">
         <v>35</v>
       </c>
-      <c r="B23" s="22"/>
-      <c r="J23" s="6"/>
-      <c r="K23" s="6"/>
-      <c r="L23" s="6"/>
-      <c r="M23" s="6"/>
-      <c r="N23" s="6"/>
-      <c r="O23" s="15"/>
-      <c r="P23" s="16"/>
-      <c r="Q23" s="16"/>
-      <c r="R23" s="16"/>
-      <c r="S23" s="6"/>
-      <c r="T23" s="6"/>
-      <c r="U23" s="6"/>
-      <c r="V23" s="6"/>
-      <c r="W23" s="6"/>
-      <c r="X23" s="6"/>
-      <c r="Y23" s="6"/>
-      <c r="Z23" s="6"/>
-      <c r="AA23" s="6"/>
+      <c r="B23" s="19"/>
+      <c r="J23" s="5"/>
+      <c r="K23" s="5"/>
+      <c r="L23" s="5"/>
+      <c r="M23" s="5"/>
+      <c r="N23" s="5"/>
+      <c r="O23" s="14"/>
+      <c r="P23" s="15"/>
+      <c r="Q23" s="15"/>
+      <c r="R23" s="15"/>
+      <c r="S23" s="5"/>
+      <c r="T23" s="5"/>
+      <c r="U23" s="5"/>
+      <c r="V23" s="5"/>
+      <c r="W23" s="5"/>
+      <c r="X23" s="5"/>
+      <c r="Y23" s="5"/>
+      <c r="Z23" s="5"/>
+      <c r="AA23" s="5"/>
     </row>
     <row r="24" spans="1:40" x14ac:dyDescent="0.4">
       <c r="A24" s="1" t="s">
@@ -1431,57 +1522,69 @@
       <c r="C24" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="O24" s="15"/>
-      <c r="P24" s="15"/>
-      <c r="Q24" s="15"/>
-      <c r="R24" s="15"/>
+      <c r="O24" s="14"/>
+      <c r="P24" s="14"/>
+      <c r="Q24" s="14"/>
+      <c r="R24" s="14"/>
     </row>
     <row r="25" spans="1:40" x14ac:dyDescent="0.4">
-      <c r="A25" s="20" t="s">
+      <c r="A25" s="17" t="s">
         <v>37</v>
       </c>
-      <c r="B25" s="20"/>
+      <c r="B25" s="17"/>
       <c r="C25" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="O25" s="15"/>
-      <c r="P25" s="15"/>
-      <c r="Q25" s="15"/>
-      <c r="R25" s="15"/>
+      <c r="O25" s="14"/>
+      <c r="P25" s="14"/>
+      <c r="Q25" s="14"/>
+      <c r="R25" s="14"/>
     </row>
     <row r="26" spans="1:40" x14ac:dyDescent="0.4">
-      <c r="A26" s="20" t="s">
+      <c r="A26" s="17" t="s">
         <v>38</v>
       </c>
-      <c r="B26" s="20"/>
+      <c r="B26" s="17"/>
       <c r="C26" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="O26" s="15"/>
-      <c r="P26" s="15"/>
-      <c r="Q26" s="15"/>
-      <c r="R26" s="15"/>
+      <c r="O26" s="14"/>
+      <c r="P26" s="14"/>
+      <c r="Q26" s="14"/>
+      <c r="R26" s="14"/>
     </row>
     <row r="27" spans="1:40" x14ac:dyDescent="0.4">
-      <c r="A27" s="20" t="s">
+      <c r="A27" s="17" t="s">
         <v>39</v>
       </c>
-      <c r="B27" s="20"/>
+      <c r="B27" s="17"/>
       <c r="C27" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="O27" s="15"/>
-      <c r="P27" s="15"/>
-      <c r="Q27" s="15"/>
-      <c r="R27" s="15"/>
+      <c r="O27" s="14"/>
+      <c r="P27" s="14"/>
+      <c r="Q27" s="14"/>
+      <c r="R27" s="14"/>
     </row>
     <row r="28" spans="1:40" x14ac:dyDescent="0.4">
-      <c r="A28" s="20"/>
-      <c r="B28" s="20"/>
-    </row>
-    <row r="29" spans="1:40" x14ac:dyDescent="0.4">
-      <c r="A29" s="20"/>
-      <c r="B29" s="20"/>
+      <c r="A28" s="17"/>
+      <c r="B28" s="17"/>
+    </row>
+    <row r="29" spans="1:40" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A29" s="20" t="s">
+        <v>45</v>
+      </c>
+      <c r="B29" s="17"/>
+    </row>
+    <row r="30" spans="1:40" x14ac:dyDescent="0.4">
+      <c r="A30" s="3" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="31" spans="1:40" x14ac:dyDescent="0.4">
+      <c r="A31" s="3" t="s">
+        <v>47</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="52">
@@ -1540,6 +1643,7 @@
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="A1" r:id="rId1" xr:uid="{262308BA-9AEC-44C1-B6C0-92E820B5EA69}"/>
+    <hyperlink ref="A29" r:id="rId2" display="https://www.windup.live/blog/wind-speed-for-windsurfing/" xr:uid="{EEFE3A0F-6111-4E0F-8541-6FE5B1EA154F}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Refactor check_wind.jl functions and enhance documentation; add check_direction and get_recs functions
</commit_message>
<xml_diff>
--- a/data/research.xlsx
+++ b/data/research.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ninal\Desktop\projects\NinasProject\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{453C454B-18B0-4133-92D4-0CC5AACD37CC}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C9AEA15-DB88-4674-977D-D8108C37A159}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="21585" windowHeight="8820" xr2:uid="{9C4ED264-3AF9-4DAD-A95C-E7848EE8F76F}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
+    <sheet name="Tabelle2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="50">
   <si>
     <t>&gt; 95</t>
   </si>
@@ -169,6 +170,12 @@
   </si>
   <si>
     <t>If sail size is recommended for up to 12 knots and gusts are 20+ knots, they are too strong.</t>
+  </si>
+  <si>
+    <t>crossshore</t>
+  </si>
+  <si>
+    <t>angle</t>
   </si>
 </sst>
 </file>
@@ -348,24 +355,6 @@
     <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -374,20 +363,8 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -400,6 +377,36 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -744,53 +751,53 @@
       <c r="B3" s="21">
         <v>0</v>
       </c>
-      <c r="C3" s="24">
+      <c r="C3" s="44">
         <v>1</v>
       </c>
-      <c r="D3" s="24"/>
-      <c r="E3" s="24"/>
-      <c r="F3" s="24">
+      <c r="D3" s="44"/>
+      <c r="E3" s="44"/>
+      <c r="F3" s="44">
         <v>2</v>
       </c>
-      <c r="G3" s="24"/>
-      <c r="H3" s="24"/>
-      <c r="I3" s="24">
+      <c r="G3" s="44"/>
+      <c r="H3" s="44"/>
+      <c r="I3" s="44">
         <v>3</v>
       </c>
-      <c r="J3" s="24"/>
-      <c r="K3" s="24"/>
-      <c r="L3" s="24"/>
-      <c r="M3" s="24">
+      <c r="J3" s="44"/>
+      <c r="K3" s="44"/>
+      <c r="L3" s="44"/>
+      <c r="M3" s="44">
         <v>4</v>
       </c>
-      <c r="N3" s="24"/>
-      <c r="O3" s="24"/>
-      <c r="P3" s="24"/>
-      <c r="Q3" s="24"/>
-      <c r="R3" s="24"/>
-      <c r="S3" s="24">
+      <c r="N3" s="44"/>
+      <c r="O3" s="44"/>
+      <c r="P3" s="44"/>
+      <c r="Q3" s="44"/>
+      <c r="R3" s="44"/>
+      <c r="S3" s="44">
         <v>5</v>
       </c>
-      <c r="T3" s="24"/>
-      <c r="U3" s="24"/>
-      <c r="V3" s="24"/>
-      <c r="W3" s="24"/>
-      <c r="X3" s="24">
+      <c r="T3" s="44"/>
+      <c r="U3" s="44"/>
+      <c r="V3" s="44"/>
+      <c r="W3" s="44"/>
+      <c r="X3" s="44">
         <v>6</v>
       </c>
-      <c r="Y3" s="24"/>
-      <c r="Z3" s="24"/>
-      <c r="AA3" s="24"/>
-      <c r="AB3" s="24"/>
-      <c r="AC3" s="24"/>
-      <c r="AD3" s="24">
+      <c r="Y3" s="44"/>
+      <c r="Z3" s="44"/>
+      <c r="AA3" s="44"/>
+      <c r="AB3" s="44"/>
+      <c r="AC3" s="44"/>
+      <c r="AD3" s="44">
         <v>7</v>
       </c>
-      <c r="AE3" s="24"/>
-      <c r="AF3" s="24"/>
-      <c r="AG3" s="24"/>
-      <c r="AH3" s="24"/>
-      <c r="AI3" s="24"/>
+      <c r="AE3" s="44"/>
+      <c r="AF3" s="44"/>
+      <c r="AG3" s="44"/>
+      <c r="AH3" s="44"/>
+      <c r="AI3" s="44"/>
       <c r="AK3" s="7" t="s">
         <v>4</v>
       </c>
@@ -910,39 +917,39 @@
         <v>9</v>
       </c>
       <c r="B5" s="22"/>
-      <c r="C5" s="23"/>
-      <c r="D5" s="23"/>
-      <c r="E5" s="23"/>
-      <c r="F5" s="25"/>
-      <c r="G5" s="25"/>
-      <c r="H5" s="25"/>
-      <c r="I5" s="26"/>
-      <c r="J5" s="26"/>
-      <c r="K5" s="26"/>
-      <c r="L5" s="26"/>
-      <c r="M5" s="28"/>
-      <c r="N5" s="28"/>
-      <c r="O5" s="28"/>
-      <c r="P5" s="28"/>
-      <c r="Q5" s="28"/>
-      <c r="R5" s="28"/>
-      <c r="S5" s="27"/>
-      <c r="T5" s="27"/>
-      <c r="U5" s="27"/>
-      <c r="V5" s="27"/>
-      <c r="W5" s="27"/>
-      <c r="X5" s="27"/>
-      <c r="Y5" s="27"/>
-      <c r="Z5" s="27"/>
-      <c r="AA5" s="27"/>
-      <c r="AB5" s="27"/>
-      <c r="AC5" s="27"/>
-      <c r="AD5" s="27"/>
-      <c r="AE5" s="27"/>
-      <c r="AF5" s="27"/>
-      <c r="AG5" s="27"/>
-      <c r="AH5" s="27"/>
-      <c r="AI5" s="27"/>
+      <c r="C5" s="43"/>
+      <c r="D5" s="43"/>
+      <c r="E5" s="43"/>
+      <c r="F5" s="42"/>
+      <c r="G5" s="42"/>
+      <c r="H5" s="42"/>
+      <c r="I5" s="41"/>
+      <c r="J5" s="41"/>
+      <c r="K5" s="41"/>
+      <c r="L5" s="41"/>
+      <c r="M5" s="40"/>
+      <c r="N5" s="40"/>
+      <c r="O5" s="40"/>
+      <c r="P5" s="40"/>
+      <c r="Q5" s="40"/>
+      <c r="R5" s="40"/>
+      <c r="S5" s="39"/>
+      <c r="T5" s="39"/>
+      <c r="U5" s="39"/>
+      <c r="V5" s="39"/>
+      <c r="W5" s="39"/>
+      <c r="X5" s="39"/>
+      <c r="Y5" s="39"/>
+      <c r="Z5" s="39"/>
+      <c r="AA5" s="39"/>
+      <c r="AB5" s="39"/>
+      <c r="AC5" s="39"/>
+      <c r="AD5" s="39"/>
+      <c r="AE5" s="39"/>
+      <c r="AF5" s="39"/>
+      <c r="AG5" s="39"/>
+      <c r="AH5" s="39"/>
+      <c r="AI5" s="39"/>
       <c r="AK5" s="9" t="s">
         <v>6</v>
       </c>
@@ -952,39 +959,39 @@
         <v>10</v>
       </c>
       <c r="B6" s="22"/>
-      <c r="C6" s="23"/>
-      <c r="D6" s="23"/>
-      <c r="E6" s="23"/>
-      <c r="F6" s="23"/>
-      <c r="G6" s="23"/>
-      <c r="H6" s="23"/>
-      <c r="I6" s="25"/>
-      <c r="J6" s="25"/>
-      <c r="K6" s="25"/>
-      <c r="L6" s="25"/>
-      <c r="M6" s="26"/>
-      <c r="N6" s="26"/>
-      <c r="O6" s="26"/>
-      <c r="P6" s="26"/>
-      <c r="Q6" s="26"/>
-      <c r="R6" s="26"/>
-      <c r="S6" s="28"/>
-      <c r="T6" s="28"/>
-      <c r="U6" s="28"/>
-      <c r="V6" s="28"/>
-      <c r="W6" s="28"/>
-      <c r="X6" s="27"/>
-      <c r="Y6" s="27"/>
-      <c r="Z6" s="27"/>
-      <c r="AA6" s="27"/>
-      <c r="AB6" s="27"/>
-      <c r="AC6" s="27"/>
-      <c r="AD6" s="27"/>
-      <c r="AE6" s="27"/>
-      <c r="AF6" s="27"/>
-      <c r="AG6" s="27"/>
-      <c r="AH6" s="27"/>
-      <c r="AI6" s="27"/>
+      <c r="C6" s="43"/>
+      <c r="D6" s="43"/>
+      <c r="E6" s="43"/>
+      <c r="F6" s="43"/>
+      <c r="G6" s="43"/>
+      <c r="H6" s="43"/>
+      <c r="I6" s="42"/>
+      <c r="J6" s="42"/>
+      <c r="K6" s="42"/>
+      <c r="L6" s="42"/>
+      <c r="M6" s="41"/>
+      <c r="N6" s="41"/>
+      <c r="O6" s="41"/>
+      <c r="P6" s="41"/>
+      <c r="Q6" s="41"/>
+      <c r="R6" s="41"/>
+      <c r="S6" s="40"/>
+      <c r="T6" s="40"/>
+      <c r="U6" s="40"/>
+      <c r="V6" s="40"/>
+      <c r="W6" s="40"/>
+      <c r="X6" s="39"/>
+      <c r="Y6" s="39"/>
+      <c r="Z6" s="39"/>
+      <c r="AA6" s="39"/>
+      <c r="AB6" s="39"/>
+      <c r="AC6" s="39"/>
+      <c r="AD6" s="39"/>
+      <c r="AE6" s="39"/>
+      <c r="AF6" s="39"/>
+      <c r="AG6" s="39"/>
+      <c r="AH6" s="39"/>
+      <c r="AI6" s="39"/>
       <c r="AJ6" s="4"/>
       <c r="AK6" s="10" t="s">
         <v>7</v>
@@ -995,116 +1002,116 @@
         <v>11</v>
       </c>
       <c r="B7" s="22"/>
-      <c r="C7" s="23"/>
-      <c r="D7" s="23"/>
-      <c r="E7" s="23"/>
-      <c r="F7" s="23"/>
-      <c r="G7" s="23"/>
-      <c r="H7" s="23"/>
-      <c r="I7" s="25"/>
-      <c r="J7" s="25"/>
-      <c r="K7" s="25"/>
-      <c r="L7" s="25"/>
-      <c r="M7" s="25"/>
-      <c r="N7" s="25"/>
-      <c r="O7" s="25"/>
-      <c r="P7" s="25"/>
-      <c r="Q7" s="25"/>
-      <c r="R7" s="25"/>
-      <c r="S7" s="26"/>
-      <c r="T7" s="26"/>
-      <c r="U7" s="26"/>
-      <c r="V7" s="26"/>
-      <c r="W7" s="26"/>
-      <c r="X7" s="28"/>
-      <c r="Y7" s="28"/>
-      <c r="Z7" s="28"/>
-      <c r="AA7" s="28"/>
-      <c r="AB7" s="28"/>
-      <c r="AC7" s="28"/>
-      <c r="AD7" s="27"/>
-      <c r="AE7" s="27"/>
-      <c r="AF7" s="27"/>
-      <c r="AG7" s="27"/>
-      <c r="AH7" s="27"/>
-      <c r="AI7" s="27"/>
+      <c r="C7" s="43"/>
+      <c r="D7" s="43"/>
+      <c r="E7" s="43"/>
+      <c r="F7" s="43"/>
+      <c r="G7" s="43"/>
+      <c r="H7" s="43"/>
+      <c r="I7" s="42"/>
+      <c r="J7" s="42"/>
+      <c r="K7" s="42"/>
+      <c r="L7" s="42"/>
+      <c r="M7" s="42"/>
+      <c r="N7" s="42"/>
+      <c r="O7" s="42"/>
+      <c r="P7" s="42"/>
+      <c r="Q7" s="42"/>
+      <c r="R7" s="42"/>
+      <c r="S7" s="41"/>
+      <c r="T7" s="41"/>
+      <c r="U7" s="41"/>
+      <c r="V7" s="41"/>
+      <c r="W7" s="41"/>
+      <c r="X7" s="40"/>
+      <c r="Y7" s="40"/>
+      <c r="Z7" s="40"/>
+      <c r="AA7" s="40"/>
+      <c r="AB7" s="40"/>
+      <c r="AC7" s="40"/>
+      <c r="AD7" s="39"/>
+      <c r="AE7" s="39"/>
+      <c r="AF7" s="39"/>
+      <c r="AG7" s="39"/>
+      <c r="AH7" s="39"/>
+      <c r="AI7" s="39"/>
       <c r="AK7" s="11" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="8" spans="1:40" x14ac:dyDescent="0.4">
-      <c r="A8" s="29" t="s">
+      <c r="A8" s="23" t="s">
         <v>32</v>
       </c>
-      <c r="B8" s="29"/>
-      <c r="C8" s="30"/>
-      <c r="D8" s="30"/>
-      <c r="E8" s="30"/>
-      <c r="F8" s="31"/>
-      <c r="G8" s="31"/>
-      <c r="H8" s="31"/>
-      <c r="I8" s="31"/>
-      <c r="J8" s="31"/>
-      <c r="K8" s="31"/>
-      <c r="L8" s="31"/>
-      <c r="M8" s="31"/>
-      <c r="N8" s="31"/>
-      <c r="O8" s="31"/>
-      <c r="P8" s="31"/>
-      <c r="Q8" s="31"/>
-      <c r="R8" s="31"/>
-      <c r="S8" s="31"/>
-      <c r="T8" s="31"/>
-      <c r="U8" s="31"/>
-      <c r="V8" s="31"/>
-      <c r="W8" s="31"/>
-      <c r="X8" s="31"/>
-      <c r="Y8" s="31"/>
-      <c r="Z8" s="31"/>
-      <c r="AA8" s="31"/>
-      <c r="AB8" s="31"/>
-      <c r="AC8" s="31"/>
-      <c r="AD8" s="31"/>
+      <c r="B8" s="23"/>
+      <c r="C8" s="24"/>
+      <c r="D8" s="24"/>
+      <c r="E8" s="24"/>
+      <c r="F8" s="25"/>
+      <c r="G8" s="25"/>
+      <c r="H8" s="25"/>
+      <c r="I8" s="25"/>
+      <c r="J8" s="25"/>
+      <c r="K8" s="25"/>
+      <c r="L8" s="25"/>
+      <c r="M8" s="25"/>
+      <c r="N8" s="25"/>
+      <c r="O8" s="25"/>
+      <c r="P8" s="25"/>
+      <c r="Q8" s="25"/>
+      <c r="R8" s="25"/>
+      <c r="S8" s="25"/>
+      <c r="T8" s="25"/>
+      <c r="U8" s="25"/>
+      <c r="V8" s="25"/>
+      <c r="W8" s="25"/>
+      <c r="X8" s="25"/>
+      <c r="Y8" s="25"/>
+      <c r="Z8" s="25"/>
+      <c r="AA8" s="25"/>
+      <c r="AB8" s="25"/>
+      <c r="AC8" s="25"/>
+      <c r="AD8" s="25"/>
     </row>
     <row r="9" spans="1:40" x14ac:dyDescent="0.4">
-      <c r="A9" s="32" t="s">
+      <c r="A9" s="26" t="s">
         <v>1</v>
       </c>
-      <c r="B9" s="32"/>
-      <c r="C9" s="30"/>
-      <c r="D9" s="30"/>
-      <c r="E9" s="30"/>
-      <c r="F9" s="31"/>
-      <c r="G9" s="30"/>
-      <c r="H9" s="30"/>
-      <c r="I9" s="33" t="s">
+      <c r="B9" s="26"/>
+      <c r="C9" s="24"/>
+      <c r="D9" s="24"/>
+      <c r="E9" s="24"/>
+      <c r="F9" s="25"/>
+      <c r="G9" s="24"/>
+      <c r="H9" s="24"/>
+      <c r="I9" s="35" t="s">
         <v>18</v>
       </c>
-      <c r="J9" s="34"/>
-      <c r="K9" s="34"/>
-      <c r="L9" s="34"/>
-      <c r="M9" s="34"/>
-      <c r="N9" s="34"/>
-      <c r="O9" s="33" t="s">
+      <c r="J9" s="36"/>
+      <c r="K9" s="36"/>
+      <c r="L9" s="36"/>
+      <c r="M9" s="36"/>
+      <c r="N9" s="36"/>
+      <c r="O9" s="35" t="s">
         <v>12</v>
       </c>
-      <c r="P9" s="34"/>
-      <c r="Q9" s="34"/>
-      <c r="R9" s="34"/>
-      <c r="S9" s="34"/>
-      <c r="T9" s="34"/>
-      <c r="U9" s="33" t="s">
+      <c r="P9" s="36"/>
+      <c r="Q9" s="36"/>
+      <c r="R9" s="36"/>
+      <c r="S9" s="36"/>
+      <c r="T9" s="36"/>
+      <c r="U9" s="35" t="s">
         <v>23</v>
       </c>
-      <c r="V9" s="34"/>
-      <c r="W9" s="34"/>
-      <c r="X9" s="34"/>
-      <c r="Y9" s="34"/>
-      <c r="Z9" s="34"/>
-      <c r="AA9" s="34"/>
-      <c r="AB9" s="34"/>
-      <c r="AC9" s="34"/>
-      <c r="AD9" s="35" t="s">
+      <c r="V9" s="36"/>
+      <c r="W9" s="36"/>
+      <c r="X9" s="36"/>
+      <c r="Y9" s="36"/>
+      <c r="Z9" s="36"/>
+      <c r="AA9" s="36"/>
+      <c r="AB9" s="36"/>
+      <c r="AC9" s="36"/>
+      <c r="AD9" s="27" t="s">
         <v>26</v>
       </c>
       <c r="AE9" s="13"/>
@@ -1115,44 +1122,44 @@
       <c r="AK9" s="16"/>
     </row>
     <row r="10" spans="1:40" x14ac:dyDescent="0.4">
-      <c r="A10" s="32" t="s">
+      <c r="A10" s="26" t="s">
         <v>14</v>
       </c>
-      <c r="B10" s="32"/>
-      <c r="C10" s="30"/>
-      <c r="D10" s="30"/>
-      <c r="E10" s="30"/>
-      <c r="F10" s="36"/>
-      <c r="G10" s="30"/>
-      <c r="H10" s="30"/>
-      <c r="I10" s="33" t="s">
+      <c r="B10" s="26"/>
+      <c r="C10" s="24"/>
+      <c r="D10" s="24"/>
+      <c r="E10" s="24"/>
+      <c r="F10" s="28"/>
+      <c r="G10" s="24"/>
+      <c r="H10" s="24"/>
+      <c r="I10" s="35" t="s">
         <v>19</v>
       </c>
-      <c r="J10" s="34"/>
-      <c r="K10" s="34"/>
-      <c r="L10" s="34"/>
-      <c r="M10" s="34"/>
-      <c r="N10" s="34"/>
-      <c r="O10" s="33" t="s">
+      <c r="J10" s="36"/>
+      <c r="K10" s="36"/>
+      <c r="L10" s="36"/>
+      <c r="M10" s="36"/>
+      <c r="N10" s="36"/>
+      <c r="O10" s="35" t="s">
         <v>18</v>
       </c>
-      <c r="P10" s="34"/>
-      <c r="Q10" s="34"/>
-      <c r="R10" s="34"/>
-      <c r="S10" s="34"/>
-      <c r="T10" s="34"/>
-      <c r="U10" s="34" t="s">
+      <c r="P10" s="36"/>
+      <c r="Q10" s="36"/>
+      <c r="R10" s="36"/>
+      <c r="S10" s="36"/>
+      <c r="T10" s="36"/>
+      <c r="U10" s="36" t="s">
         <v>12</v>
       </c>
-      <c r="V10" s="34"/>
-      <c r="W10" s="34"/>
-      <c r="X10" s="34"/>
-      <c r="Y10" s="34"/>
-      <c r="Z10" s="34"/>
-      <c r="AA10" s="34"/>
-      <c r="AB10" s="34"/>
-      <c r="AC10" s="34"/>
-      <c r="AD10" s="35" t="s">
+      <c r="V10" s="36"/>
+      <c r="W10" s="36"/>
+      <c r="X10" s="36"/>
+      <c r="Y10" s="36"/>
+      <c r="Z10" s="36"/>
+      <c r="AA10" s="36"/>
+      <c r="AB10" s="36"/>
+      <c r="AC10" s="36"/>
+      <c r="AD10" s="27" t="s">
         <v>27</v>
       </c>
       <c r="AE10" s="13"/>
@@ -1166,44 +1173,44 @@
       <c r="AN10" s="12"/>
     </row>
     <row r="11" spans="1:40" x14ac:dyDescent="0.4">
-      <c r="A11" s="32" t="s">
+      <c r="A11" s="26" t="s">
         <v>15</v>
       </c>
-      <c r="B11" s="32"/>
-      <c r="C11" s="30"/>
-      <c r="D11" s="30"/>
-      <c r="E11" s="30"/>
-      <c r="F11" s="36"/>
-      <c r="G11" s="30"/>
-      <c r="H11" s="30"/>
-      <c r="I11" s="33" t="s">
+      <c r="B11" s="26"/>
+      <c r="C11" s="24"/>
+      <c r="D11" s="24"/>
+      <c r="E11" s="24"/>
+      <c r="F11" s="28"/>
+      <c r="G11" s="24"/>
+      <c r="H11" s="24"/>
+      <c r="I11" s="35" t="s">
         <v>13</v>
       </c>
-      <c r="J11" s="34"/>
-      <c r="K11" s="34"/>
-      <c r="L11" s="34"/>
-      <c r="M11" s="34"/>
-      <c r="N11" s="34"/>
-      <c r="O11" s="33" t="s">
+      <c r="J11" s="36"/>
+      <c r="K11" s="36"/>
+      <c r="L11" s="36"/>
+      <c r="M11" s="36"/>
+      <c r="N11" s="36"/>
+      <c r="O11" s="35" t="s">
         <v>19</v>
       </c>
-      <c r="P11" s="34"/>
-      <c r="Q11" s="34"/>
-      <c r="R11" s="34"/>
-      <c r="S11" s="34"/>
-      <c r="T11" s="34"/>
-      <c r="U11" s="34" t="s">
+      <c r="P11" s="36"/>
+      <c r="Q11" s="36"/>
+      <c r="R11" s="36"/>
+      <c r="S11" s="36"/>
+      <c r="T11" s="36"/>
+      <c r="U11" s="36" t="s">
         <v>18</v>
       </c>
-      <c r="V11" s="34"/>
-      <c r="W11" s="34"/>
-      <c r="X11" s="34"/>
-      <c r="Y11" s="34"/>
-      <c r="Z11" s="34"/>
-      <c r="AA11" s="34"/>
-      <c r="AB11" s="34"/>
-      <c r="AC11" s="34"/>
-      <c r="AD11" s="35" t="s">
+      <c r="V11" s="36"/>
+      <c r="W11" s="36"/>
+      <c r="X11" s="36"/>
+      <c r="Y11" s="36"/>
+      <c r="Z11" s="36"/>
+      <c r="AA11" s="36"/>
+      <c r="AB11" s="36"/>
+      <c r="AC11" s="36"/>
+      <c r="AD11" s="27" t="s">
         <v>28</v>
       </c>
       <c r="AE11" s="13"/>
@@ -1214,16 +1221,16 @@
       <c r="AK11" s="14"/>
     </row>
     <row r="12" spans="1:40" x14ac:dyDescent="0.4">
-      <c r="A12" s="32" t="s">
+      <c r="A12" s="26" t="s">
         <v>16</v>
       </c>
-      <c r="B12" s="32"/>
-      <c r="C12" s="30"/>
-      <c r="D12" s="30"/>
-      <c r="E12" s="30"/>
-      <c r="F12" s="36"/>
-      <c r="G12" s="30"/>
-      <c r="H12" s="30"/>
+      <c r="B12" s="26"/>
+      <c r="C12" s="24"/>
+      <c r="D12" s="24"/>
+      <c r="E12" s="24"/>
+      <c r="F12" s="28"/>
+      <c r="G12" s="24"/>
+      <c r="H12" s="24"/>
       <c r="I12" s="37" t="s">
         <v>21</v>
       </c>
@@ -1232,26 +1239,26 @@
       <c r="L12" s="38"/>
       <c r="M12" s="38"/>
       <c r="N12" s="38"/>
-      <c r="O12" s="33" t="s">
+      <c r="O12" s="35" t="s">
         <v>13</v>
       </c>
-      <c r="P12" s="34"/>
-      <c r="Q12" s="34"/>
-      <c r="R12" s="34"/>
-      <c r="S12" s="34"/>
-      <c r="T12" s="34"/>
-      <c r="U12" s="34" t="s">
+      <c r="P12" s="36"/>
+      <c r="Q12" s="36"/>
+      <c r="R12" s="36"/>
+      <c r="S12" s="36"/>
+      <c r="T12" s="36"/>
+      <c r="U12" s="36" t="s">
         <v>19</v>
       </c>
-      <c r="V12" s="34"/>
-      <c r="W12" s="34"/>
-      <c r="X12" s="34"/>
-      <c r="Y12" s="34"/>
-      <c r="Z12" s="34"/>
-      <c r="AA12" s="34"/>
-      <c r="AB12" s="34"/>
-      <c r="AC12" s="34"/>
-      <c r="AD12" s="35" t="s">
+      <c r="V12" s="36"/>
+      <c r="W12" s="36"/>
+      <c r="X12" s="36"/>
+      <c r="Y12" s="36"/>
+      <c r="Z12" s="36"/>
+      <c r="AA12" s="36"/>
+      <c r="AB12" s="36"/>
+      <c r="AC12" s="36"/>
+      <c r="AD12" s="27" t="s">
         <v>29</v>
       </c>
       <c r="AE12" s="13"/>
@@ -1262,16 +1269,16 @@
       <c r="AK12" s="14"/>
     </row>
     <row r="13" spans="1:40" x14ac:dyDescent="0.4">
-      <c r="A13" s="32" t="s">
+      <c r="A13" s="26" t="s">
         <v>17</v>
       </c>
-      <c r="B13" s="32"/>
-      <c r="C13" s="30"/>
-      <c r="D13" s="30"/>
-      <c r="E13" s="30"/>
-      <c r="F13" s="36"/>
-      <c r="G13" s="30"/>
-      <c r="H13" s="30"/>
+      <c r="B13" s="26"/>
+      <c r="C13" s="24"/>
+      <c r="D13" s="24"/>
+      <c r="E13" s="24"/>
+      <c r="F13" s="28"/>
+      <c r="G13" s="24"/>
+      <c r="H13" s="24"/>
       <c r="I13" s="37" t="s">
         <v>22</v>
       </c>
@@ -1280,26 +1287,26 @@
       <c r="L13" s="38"/>
       <c r="M13" s="38"/>
       <c r="N13" s="38"/>
-      <c r="O13" s="33" t="s">
+      <c r="O13" s="35" t="s">
         <v>21</v>
       </c>
-      <c r="P13" s="34"/>
-      <c r="Q13" s="34"/>
-      <c r="R13" s="34"/>
-      <c r="S13" s="34"/>
-      <c r="T13" s="34"/>
-      <c r="U13" s="34" t="s">
+      <c r="P13" s="36"/>
+      <c r="Q13" s="36"/>
+      <c r="R13" s="36"/>
+      <c r="S13" s="36"/>
+      <c r="T13" s="36"/>
+      <c r="U13" s="36" t="s">
         <v>13</v>
       </c>
-      <c r="V13" s="34"/>
-      <c r="W13" s="34"/>
-      <c r="X13" s="34"/>
-      <c r="Y13" s="34"/>
-      <c r="Z13" s="34"/>
-      <c r="AA13" s="34"/>
-      <c r="AB13" s="34"/>
-      <c r="AC13" s="34"/>
-      <c r="AD13" s="35" t="s">
+      <c r="V13" s="36"/>
+      <c r="W13" s="36"/>
+      <c r="X13" s="36"/>
+      <c r="Y13" s="36"/>
+      <c r="Z13" s="36"/>
+      <c r="AA13" s="36"/>
+      <c r="AB13" s="36"/>
+      <c r="AC13" s="36"/>
+      <c r="AD13" s="27" t="s">
         <v>30</v>
       </c>
       <c r="AE13" s="13"/>
@@ -1313,80 +1320,80 @@
       <c r="AN13" s="12"/>
     </row>
     <row r="14" spans="1:40" x14ac:dyDescent="0.4">
-      <c r="A14" s="32" t="s">
+      <c r="A14" s="26" t="s">
         <v>0</v>
       </c>
-      <c r="B14" s="32"/>
-      <c r="C14" s="30"/>
-      <c r="D14" s="30"/>
-      <c r="E14" s="30"/>
-      <c r="F14" s="36"/>
-      <c r="G14" s="30"/>
-      <c r="H14" s="30"/>
-      <c r="I14" s="33" t="s">
+      <c r="B14" s="26"/>
+      <c r="C14" s="24"/>
+      <c r="D14" s="24"/>
+      <c r="E14" s="24"/>
+      <c r="F14" s="28"/>
+      <c r="G14" s="24"/>
+      <c r="H14" s="24"/>
+      <c r="I14" s="35" t="s">
         <v>20</v>
       </c>
-      <c r="J14" s="34"/>
-      <c r="K14" s="34"/>
-      <c r="L14" s="34"/>
-      <c r="M14" s="34"/>
-      <c r="N14" s="34"/>
-      <c r="O14" s="33" t="s">
+      <c r="J14" s="36"/>
+      <c r="K14" s="36"/>
+      <c r="L14" s="36"/>
+      <c r="M14" s="36"/>
+      <c r="N14" s="36"/>
+      <c r="O14" s="35" t="s">
         <v>22</v>
       </c>
-      <c r="P14" s="34"/>
-      <c r="Q14" s="34"/>
-      <c r="R14" s="34"/>
-      <c r="S14" s="34"/>
-      <c r="T14" s="34"/>
-      <c r="U14" s="34" t="s">
+      <c r="P14" s="36"/>
+      <c r="Q14" s="36"/>
+      <c r="R14" s="36"/>
+      <c r="S14" s="36"/>
+      <c r="T14" s="36"/>
+      <c r="U14" s="36" t="s">
         <v>21</v>
       </c>
-      <c r="V14" s="34"/>
-      <c r="W14" s="34"/>
-      <c r="X14" s="34"/>
-      <c r="Y14" s="34"/>
-      <c r="Z14" s="34"/>
-      <c r="AA14" s="34"/>
-      <c r="AB14" s="34"/>
-      <c r="AC14" s="34"/>
-      <c r="AD14" s="31"/>
+      <c r="V14" s="36"/>
+      <c r="W14" s="36"/>
+      <c r="X14" s="36"/>
+      <c r="Y14" s="36"/>
+      <c r="Z14" s="36"/>
+      <c r="AA14" s="36"/>
+      <c r="AB14" s="36"/>
+      <c r="AC14" s="36"/>
+      <c r="AD14" s="25"/>
     </row>
     <row r="15" spans="1:40" x14ac:dyDescent="0.4">
-      <c r="A15" s="39" t="s">
+      <c r="A15" s="29" t="s">
         <v>34</v>
       </c>
-      <c r="B15" s="39"/>
-      <c r="C15" s="40"/>
-      <c r="D15" s="40"/>
-      <c r="E15" s="40"/>
-      <c r="F15" s="41"/>
+      <c r="B15" s="29"/>
+      <c r="C15" s="30"/>
+      <c r="D15" s="30"/>
+      <c r="E15" s="30"/>
+      <c r="F15" s="31"/>
       <c r="AL15" s="12"/>
       <c r="AM15" s="12"/>
       <c r="AN15" s="12"/>
     </row>
     <row r="16" spans="1:40" x14ac:dyDescent="0.4">
-      <c r="A16" s="42" t="s">
+      <c r="A16" s="32" t="s">
         <v>24</v>
       </c>
-      <c r="B16" s="42"/>
-      <c r="C16" s="40"/>
-      <c r="D16" s="40"/>
-      <c r="E16" s="40"/>
-      <c r="F16" s="41"/>
+      <c r="B16" s="32"/>
+      <c r="C16" s="30"/>
+      <c r="D16" s="30"/>
+      <c r="E16" s="30"/>
+      <c r="F16" s="31"/>
     </row>
     <row r="17" spans="1:40" x14ac:dyDescent="0.4">
-      <c r="A17" s="43" t="s">
+      <c r="A17" s="33" t="s">
         <v>1</v>
       </c>
-      <c r="B17" s="43"/>
-      <c r="C17" s="44">
+      <c r="B17" s="33"/>
+      <c r="C17" s="34">
         <f>55/15</f>
         <v>3.6666666666666665</v>
       </c>
-      <c r="D17" s="44"/>
-      <c r="E17" s="44"/>
-      <c r="F17" s="41" t="s">
+      <c r="D17" s="34"/>
+      <c r="E17" s="34"/>
+      <c r="F17" s="31" t="s">
         <v>25</v>
       </c>
       <c r="AL17" s="12"/>
@@ -1394,83 +1401,83 @@
       <c r="AN17" s="12"/>
     </row>
     <row r="18" spans="1:40" x14ac:dyDescent="0.4">
-      <c r="A18" s="43" t="s">
+      <c r="A18" s="33" t="s">
         <v>14</v>
       </c>
-      <c r="B18" s="43"/>
-      <c r="C18" s="44">
+      <c r="B18" s="33"/>
+      <c r="C18" s="34">
         <f>65/15</f>
         <v>4.333333333333333</v>
       </c>
-      <c r="D18" s="44"/>
-      <c r="E18" s="44"/>
-      <c r="F18" s="41" t="s">
+      <c r="D18" s="34"/>
+      <c r="E18" s="34"/>
+      <c r="F18" s="31" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="19" spans="1:40" x14ac:dyDescent="0.4">
-      <c r="A19" s="43" t="s">
+      <c r="A19" s="33" t="s">
         <v>15</v>
       </c>
-      <c r="B19" s="43"/>
-      <c r="C19" s="44">
+      <c r="B19" s="33"/>
+      <c r="C19" s="34">
         <f>75/15</f>
         <v>5</v>
       </c>
-      <c r="D19" s="44"/>
-      <c r="E19" s="44"/>
-      <c r="F19" s="41"/>
+      <c r="D19" s="34"/>
+      <c r="E19" s="34"/>
+      <c r="F19" s="31"/>
       <c r="O19" s="14"/>
       <c r="P19" s="14"/>
       <c r="Q19" s="14"/>
       <c r="R19" s="14"/>
     </row>
     <row r="20" spans="1:40" x14ac:dyDescent="0.4">
-      <c r="A20" s="43" t="s">
+      <c r="A20" s="33" t="s">
         <v>16</v>
       </c>
-      <c r="B20" s="43"/>
-      <c r="C20" s="44">
+      <c r="B20" s="33"/>
+      <c r="C20" s="34">
         <f>85/15</f>
         <v>5.666666666666667</v>
       </c>
-      <c r="D20" s="44"/>
-      <c r="E20" s="44"/>
-      <c r="F20" s="41"/>
+      <c r="D20" s="34"/>
+      <c r="E20" s="34"/>
+      <c r="F20" s="31"/>
       <c r="O20" s="14"/>
       <c r="P20" s="14"/>
       <c r="Q20" s="14"/>
       <c r="R20" s="14"/>
     </row>
     <row r="21" spans="1:40" x14ac:dyDescent="0.4">
-      <c r="A21" s="43" t="s">
+      <c r="A21" s="33" t="s">
         <v>17</v>
       </c>
-      <c r="B21" s="43"/>
-      <c r="C21" s="44">
+      <c r="B21" s="33"/>
+      <c r="C21" s="34">
         <f>95/15</f>
         <v>6.333333333333333</v>
       </c>
-      <c r="D21" s="44"/>
-      <c r="E21" s="44"/>
-      <c r="F21" s="41"/>
+      <c r="D21" s="34"/>
+      <c r="E21" s="34"/>
+      <c r="F21" s="31"/>
       <c r="O21" s="14"/>
       <c r="P21" s="14"/>
       <c r="Q21" s="14"/>
       <c r="R21" s="14"/>
     </row>
     <row r="22" spans="1:40" x14ac:dyDescent="0.4">
-      <c r="A22" s="43" t="s">
+      <c r="A22" s="33" t="s">
         <v>0</v>
       </c>
-      <c r="B22" s="43"/>
-      <c r="C22" s="44">
+      <c r="B22" s="33"/>
+      <c r="C22" s="34">
         <f>105/15</f>
         <v>7</v>
       </c>
-      <c r="D22" s="44"/>
-      <c r="E22" s="44"/>
-      <c r="F22" s="41"/>
+      <c r="D22" s="34"/>
+      <c r="E22" s="34"/>
+      <c r="F22" s="31"/>
       <c r="J22" s="5"/>
       <c r="K22" s="5"/>
       <c r="L22" s="5"/>
@@ -1588,26 +1595,22 @@
     </row>
   </sheetData>
   <mergeCells count="52">
-    <mergeCell ref="C22:E22"/>
-    <mergeCell ref="I9:N9"/>
-    <mergeCell ref="I10:N10"/>
-    <mergeCell ref="I11:N11"/>
-    <mergeCell ref="I12:N12"/>
-    <mergeCell ref="I13:N13"/>
-    <mergeCell ref="I14:N14"/>
-    <mergeCell ref="O9:T9"/>
-    <mergeCell ref="O10:T10"/>
-    <mergeCell ref="C21:E21"/>
-    <mergeCell ref="C17:E17"/>
-    <mergeCell ref="C18:E18"/>
-    <mergeCell ref="C19:E19"/>
-    <mergeCell ref="C20:E20"/>
-    <mergeCell ref="U13:AC13"/>
-    <mergeCell ref="AD7:AI7"/>
-    <mergeCell ref="AD6:AI6"/>
-    <mergeCell ref="AD5:AI5"/>
-    <mergeCell ref="X7:AC7"/>
-    <mergeCell ref="U9:AC9"/>
+    <mergeCell ref="C7:E7"/>
+    <mergeCell ref="C5:E5"/>
+    <mergeCell ref="AD3:AI3"/>
+    <mergeCell ref="C6:E6"/>
+    <mergeCell ref="C3:E3"/>
+    <mergeCell ref="F3:H3"/>
+    <mergeCell ref="I3:L3"/>
+    <mergeCell ref="M3:R3"/>
+    <mergeCell ref="S3:W3"/>
+    <mergeCell ref="X3:AC3"/>
+    <mergeCell ref="I7:L7"/>
+    <mergeCell ref="I6:L6"/>
+    <mergeCell ref="I5:L5"/>
+    <mergeCell ref="F7:H7"/>
+    <mergeCell ref="F6:H6"/>
+    <mergeCell ref="F5:H5"/>
     <mergeCell ref="U14:AC14"/>
     <mergeCell ref="X5:AC5"/>
     <mergeCell ref="S7:W7"/>
@@ -1624,22 +1627,26 @@
     <mergeCell ref="U11:AC11"/>
     <mergeCell ref="U12:AC12"/>
     <mergeCell ref="X6:AC6"/>
-    <mergeCell ref="C7:E7"/>
-    <mergeCell ref="C5:E5"/>
-    <mergeCell ref="AD3:AI3"/>
-    <mergeCell ref="C6:E6"/>
-    <mergeCell ref="C3:E3"/>
-    <mergeCell ref="F3:H3"/>
-    <mergeCell ref="I3:L3"/>
-    <mergeCell ref="M3:R3"/>
-    <mergeCell ref="S3:W3"/>
-    <mergeCell ref="X3:AC3"/>
-    <mergeCell ref="I7:L7"/>
-    <mergeCell ref="I6:L6"/>
-    <mergeCell ref="I5:L5"/>
-    <mergeCell ref="F7:H7"/>
-    <mergeCell ref="F6:H6"/>
-    <mergeCell ref="F5:H5"/>
+    <mergeCell ref="U13:AC13"/>
+    <mergeCell ref="AD7:AI7"/>
+    <mergeCell ref="AD6:AI6"/>
+    <mergeCell ref="AD5:AI5"/>
+    <mergeCell ref="X7:AC7"/>
+    <mergeCell ref="U9:AC9"/>
+    <mergeCell ref="O9:T9"/>
+    <mergeCell ref="O10:T10"/>
+    <mergeCell ref="C21:E21"/>
+    <mergeCell ref="C17:E17"/>
+    <mergeCell ref="C18:E18"/>
+    <mergeCell ref="C19:E19"/>
+    <mergeCell ref="C20:E20"/>
+    <mergeCell ref="C22:E22"/>
+    <mergeCell ref="I9:N9"/>
+    <mergeCell ref="I10:N10"/>
+    <mergeCell ref="I11:N11"/>
+    <mergeCell ref="I12:N12"/>
+    <mergeCell ref="I13:N13"/>
+    <mergeCell ref="I14:N14"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="A1" r:id="rId1" xr:uid="{262308BA-9AEC-44C1-B6C0-92E820B5EA69}"/>
@@ -1647,4 +1654,100 @@
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B5FAFDF3-FEFD-4C1F-A721-3F22A7C4179E}">
+  <dimension ref="A1:C8"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <cols>
+    <col min="1" max="1" width="13.06640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A1" t="s">
+        <v>49</v>
+      </c>
+      <c r="B1">
+        <f>270</f>
+        <v>270</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A3" t="s">
+        <v>37</v>
+      </c>
+      <c r="B3">
+        <f>IF($B$1+110&gt;360, $B$1+110-360,$B$1+110)</f>
+        <v>20</v>
+      </c>
+      <c r="C3">
+        <f>IF($B$1-110&lt;=0, $B$1-110+360,$B$1-110)</f>
+        <v>160</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A4" t="s">
+        <v>48</v>
+      </c>
+      <c r="B4">
+        <f>IF($B$1+67.5&gt;360, $B$1+67.5-360,$B$1+67.5)</f>
+        <v>337.5</v>
+      </c>
+      <c r="C4">
+        <f>IF($B$1+110&gt;360, $B$1+110-360,$B$1+110)</f>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A5" t="s">
+        <v>39</v>
+      </c>
+      <c r="B5">
+        <f>IF($B$1+22.5&gt;360, $B$1+22.5-360,$B$1+22.5)</f>
+        <v>292.5</v>
+      </c>
+      <c r="C5">
+        <f>IF($B$1+67.5&gt;360, $B$1+67.5-360,$B$1+67.5)</f>
+        <v>337.5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A6" t="s">
+        <v>36</v>
+      </c>
+      <c r="B6">
+        <v>247.5</v>
+      </c>
+      <c r="C6">
+        <f>IF($B$1+22.5&gt;360, $B$1+22.5-360,$B$1+22.5)</f>
+        <v>292.5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A7" t="s">
+        <v>39</v>
+      </c>
+      <c r="B7">
+        <v>202.5</v>
+      </c>
+      <c r="C7">
+        <v>247.5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A8" t="s">
+        <v>48</v>
+      </c>
+      <c r="B8">
+        <v>160</v>
+      </c>
+      <c r="C8">
+        <v>202.5</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Correct mistakes in the guidelines
</commit_message>
<xml_diff>
--- a/data/research.xlsx
+++ b/data/research.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ninal\Desktop\projects\NinasProject\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C9AEA15-DB88-4674-977D-D8108C37A159}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7DD975B-9769-4BF6-9EB8-60E0CF443783}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="21585" windowHeight="8820" xr2:uid="{9C4ED264-3AF9-4DAD-A95C-E7848EE8F76F}"/>
   </bookViews>
@@ -307,7 +307,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -364,7 +364,6 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -376,37 +375,34 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="7" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -751,53 +747,53 @@
       <c r="B3" s="21">
         <v>0</v>
       </c>
-      <c r="C3" s="44">
+      <c r="C3" s="34">
         <v>1</v>
       </c>
-      <c r="D3" s="44"/>
-      <c r="E3" s="44"/>
-      <c r="F3" s="44">
+      <c r="D3" s="34"/>
+      <c r="E3" s="34"/>
+      <c r="F3" s="34">
         <v>2</v>
       </c>
-      <c r="G3" s="44"/>
-      <c r="H3" s="44"/>
-      <c r="I3" s="44">
+      <c r="G3" s="34"/>
+      <c r="H3" s="34"/>
+      <c r="I3" s="34">
         <v>3</v>
       </c>
-      <c r="J3" s="44"/>
-      <c r="K3" s="44"/>
-      <c r="L3" s="44"/>
-      <c r="M3" s="44">
+      <c r="J3" s="34"/>
+      <c r="K3" s="34"/>
+      <c r="L3" s="34"/>
+      <c r="M3" s="34">
         <v>4</v>
       </c>
-      <c r="N3" s="44"/>
-      <c r="O3" s="44"/>
-      <c r="P3" s="44"/>
-      <c r="Q3" s="44"/>
-      <c r="R3" s="44"/>
-      <c r="S3" s="44">
+      <c r="N3" s="34"/>
+      <c r="O3" s="34"/>
+      <c r="P3" s="34"/>
+      <c r="Q3" s="34"/>
+      <c r="R3" s="34"/>
+      <c r="S3" s="34">
         <v>5</v>
       </c>
-      <c r="T3" s="44"/>
-      <c r="U3" s="44"/>
-      <c r="V3" s="44"/>
-      <c r="W3" s="44"/>
-      <c r="X3" s="44">
+      <c r="T3" s="34"/>
+      <c r="U3" s="34"/>
+      <c r="V3" s="34"/>
+      <c r="W3" s="34"/>
+      <c r="X3" s="34">
         <v>6</v>
       </c>
-      <c r="Y3" s="44"/>
-      <c r="Z3" s="44"/>
-      <c r="AA3" s="44"/>
-      <c r="AB3" s="44"/>
-      <c r="AC3" s="44"/>
-      <c r="AD3" s="44">
+      <c r="Y3" s="34"/>
+      <c r="Z3" s="34"/>
+      <c r="AA3" s="34"/>
+      <c r="AB3" s="34"/>
+      <c r="AC3" s="34"/>
+      <c r="AD3" s="34">
         <v>7</v>
       </c>
-      <c r="AE3" s="44"/>
-      <c r="AF3" s="44"/>
-      <c r="AG3" s="44"/>
-      <c r="AH3" s="44"/>
-      <c r="AI3" s="44"/>
+      <c r="AE3" s="34"/>
+      <c r="AF3" s="34"/>
+      <c r="AG3" s="34"/>
+      <c r="AH3" s="34"/>
+      <c r="AI3" s="34"/>
       <c r="AK3" s="7" t="s">
         <v>4</v>
       </c>
@@ -917,39 +913,39 @@
         <v>9</v>
       </c>
       <c r="B5" s="22"/>
-      <c r="C5" s="43"/>
-      <c r="D5" s="43"/>
-      <c r="E5" s="43"/>
-      <c r="F5" s="42"/>
-      <c r="G5" s="42"/>
-      <c r="H5" s="42"/>
-      <c r="I5" s="41"/>
-      <c r="J5" s="41"/>
-      <c r="K5" s="41"/>
-      <c r="L5" s="41"/>
-      <c r="M5" s="40"/>
-      <c r="N5" s="40"/>
-      <c r="O5" s="40"/>
-      <c r="P5" s="40"/>
-      <c r="Q5" s="40"/>
-      <c r="R5" s="40"/>
-      <c r="S5" s="39"/>
-      <c r="T5" s="39"/>
-      <c r="U5" s="39"/>
-      <c r="V5" s="39"/>
-      <c r="W5" s="39"/>
-      <c r="X5" s="39"/>
-      <c r="Y5" s="39"/>
-      <c r="Z5" s="39"/>
-      <c r="AA5" s="39"/>
-      <c r="AB5" s="39"/>
-      <c r="AC5" s="39"/>
-      <c r="AD5" s="39"/>
-      <c r="AE5" s="39"/>
-      <c r="AF5" s="39"/>
-      <c r="AG5" s="39"/>
-      <c r="AH5" s="39"/>
-      <c r="AI5" s="39"/>
+      <c r="C5" s="33"/>
+      <c r="D5" s="33"/>
+      <c r="E5" s="33"/>
+      <c r="F5" s="35"/>
+      <c r="G5" s="35"/>
+      <c r="H5" s="35"/>
+      <c r="I5" s="36"/>
+      <c r="J5" s="36"/>
+      <c r="K5" s="36"/>
+      <c r="L5" s="36"/>
+      <c r="M5" s="39"/>
+      <c r="N5" s="39"/>
+      <c r="O5" s="39"/>
+      <c r="P5" s="39"/>
+      <c r="Q5" s="39"/>
+      <c r="R5" s="39"/>
+      <c r="S5" s="38"/>
+      <c r="T5" s="38"/>
+      <c r="U5" s="38"/>
+      <c r="V5" s="38"/>
+      <c r="W5" s="38"/>
+      <c r="X5" s="38"/>
+      <c r="Y5" s="38"/>
+      <c r="Z5" s="38"/>
+      <c r="AA5" s="38"/>
+      <c r="AB5" s="38"/>
+      <c r="AC5" s="38"/>
+      <c r="AD5" s="38"/>
+      <c r="AE5" s="38"/>
+      <c r="AF5" s="38"/>
+      <c r="AG5" s="38"/>
+      <c r="AH5" s="38"/>
+      <c r="AI5" s="38"/>
       <c r="AK5" s="9" t="s">
         <v>6</v>
       </c>
@@ -959,39 +955,39 @@
         <v>10</v>
       </c>
       <c r="B6" s="22"/>
-      <c r="C6" s="43"/>
-      <c r="D6" s="43"/>
-      <c r="E6" s="43"/>
-      <c r="F6" s="43"/>
-      <c r="G6" s="43"/>
-      <c r="H6" s="43"/>
-      <c r="I6" s="42"/>
-      <c r="J6" s="42"/>
-      <c r="K6" s="42"/>
-      <c r="L6" s="42"/>
-      <c r="M6" s="41"/>
-      <c r="N6" s="41"/>
-      <c r="O6" s="41"/>
-      <c r="P6" s="41"/>
-      <c r="Q6" s="41"/>
-      <c r="R6" s="41"/>
-      <c r="S6" s="40"/>
-      <c r="T6" s="40"/>
-      <c r="U6" s="40"/>
-      <c r="V6" s="40"/>
-      <c r="W6" s="40"/>
-      <c r="X6" s="39"/>
-      <c r="Y6" s="39"/>
-      <c r="Z6" s="39"/>
-      <c r="AA6" s="39"/>
-      <c r="AB6" s="39"/>
-      <c r="AC6" s="39"/>
-      <c r="AD6" s="39"/>
-      <c r="AE6" s="39"/>
-      <c r="AF6" s="39"/>
-      <c r="AG6" s="39"/>
-      <c r="AH6" s="39"/>
-      <c r="AI6" s="39"/>
+      <c r="C6" s="33"/>
+      <c r="D6" s="33"/>
+      <c r="E6" s="33"/>
+      <c r="F6" s="33"/>
+      <c r="G6" s="33"/>
+      <c r="H6" s="33"/>
+      <c r="I6" s="35"/>
+      <c r="J6" s="35"/>
+      <c r="K6" s="35"/>
+      <c r="L6" s="35"/>
+      <c r="M6" s="36"/>
+      <c r="N6" s="36"/>
+      <c r="O6" s="36"/>
+      <c r="P6" s="36"/>
+      <c r="Q6" s="36"/>
+      <c r="R6" s="36"/>
+      <c r="S6" s="39"/>
+      <c r="T6" s="39"/>
+      <c r="U6" s="39"/>
+      <c r="V6" s="39"/>
+      <c r="W6" s="39"/>
+      <c r="X6" s="38"/>
+      <c r="Y6" s="38"/>
+      <c r="Z6" s="38"/>
+      <c r="AA6" s="38"/>
+      <c r="AB6" s="38"/>
+      <c r="AC6" s="38"/>
+      <c r="AD6" s="38"/>
+      <c r="AE6" s="38"/>
+      <c r="AF6" s="38"/>
+      <c r="AG6" s="38"/>
+      <c r="AH6" s="38"/>
+      <c r="AI6" s="38"/>
       <c r="AJ6" s="4"/>
       <c r="AK6" s="10" t="s">
         <v>7</v>
@@ -1002,39 +998,39 @@
         <v>11</v>
       </c>
       <c r="B7" s="22"/>
-      <c r="C7" s="43"/>
-      <c r="D7" s="43"/>
-      <c r="E7" s="43"/>
-      <c r="F7" s="43"/>
-      <c r="G7" s="43"/>
-      <c r="H7" s="43"/>
-      <c r="I7" s="42"/>
-      <c r="J7" s="42"/>
-      <c r="K7" s="42"/>
-      <c r="L7" s="42"/>
-      <c r="M7" s="42"/>
-      <c r="N7" s="42"/>
-      <c r="O7" s="42"/>
-      <c r="P7" s="42"/>
-      <c r="Q7" s="42"/>
-      <c r="R7" s="42"/>
-      <c r="S7" s="41"/>
-      <c r="T7" s="41"/>
-      <c r="U7" s="41"/>
-      <c r="V7" s="41"/>
-      <c r="W7" s="41"/>
-      <c r="X7" s="40"/>
-      <c r="Y7" s="40"/>
-      <c r="Z7" s="40"/>
-      <c r="AA7" s="40"/>
-      <c r="AB7" s="40"/>
-      <c r="AC7" s="40"/>
-      <c r="AD7" s="39"/>
-      <c r="AE7" s="39"/>
-      <c r="AF7" s="39"/>
-      <c r="AG7" s="39"/>
-      <c r="AH7" s="39"/>
-      <c r="AI7" s="39"/>
+      <c r="C7" s="33"/>
+      <c r="D7" s="33"/>
+      <c r="E7" s="33"/>
+      <c r="F7" s="33"/>
+      <c r="G7" s="33"/>
+      <c r="H7" s="33"/>
+      <c r="I7" s="35"/>
+      <c r="J7" s="35"/>
+      <c r="K7" s="35"/>
+      <c r="L7" s="35"/>
+      <c r="M7" s="35"/>
+      <c r="N7" s="35"/>
+      <c r="O7" s="35"/>
+      <c r="P7" s="35"/>
+      <c r="Q7" s="35"/>
+      <c r="R7" s="35"/>
+      <c r="S7" s="36"/>
+      <c r="T7" s="36"/>
+      <c r="U7" s="36"/>
+      <c r="V7" s="36"/>
+      <c r="W7" s="36"/>
+      <c r="X7" s="39"/>
+      <c r="Y7" s="39"/>
+      <c r="Z7" s="39"/>
+      <c r="AA7" s="39"/>
+      <c r="AB7" s="39"/>
+      <c r="AC7" s="39"/>
+      <c r="AD7" s="38"/>
+      <c r="AE7" s="38"/>
+      <c r="AF7" s="38"/>
+      <c r="AG7" s="38"/>
+      <c r="AH7" s="38"/>
+      <c r="AI7" s="38"/>
       <c r="AK7" s="11" t="s">
         <v>8</v>
       </c>
@@ -1073,7 +1069,7 @@
       <c r="AC8" s="25"/>
       <c r="AD8" s="25"/>
     </row>
-    <row r="9" spans="1:40" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:40" ht="14.25" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A9" s="26" t="s">
         <v>1</v>
       </c>
@@ -1081,36 +1077,36 @@
       <c r="C9" s="24"/>
       <c r="D9" s="24"/>
       <c r="E9" s="24"/>
-      <c r="F9" s="25"/>
-      <c r="G9" s="24"/>
-      <c r="H9" s="24"/>
-      <c r="I9" s="35" t="s">
+      <c r="F9" s="40" t="s">
         <v>18</v>
       </c>
-      <c r="J9" s="36"/>
-      <c r="K9" s="36"/>
-      <c r="L9" s="36"/>
-      <c r="M9" s="36"/>
-      <c r="N9" s="36"/>
-      <c r="O9" s="35" t="s">
+      <c r="G9" s="40"/>
+      <c r="H9" s="40"/>
+      <c r="I9" s="40"/>
+      <c r="J9" s="40"/>
+      <c r="K9" s="40"/>
+      <c r="L9" s="40"/>
+      <c r="M9" s="40"/>
+      <c r="N9" s="40"/>
+      <c r="O9" s="40" t="s">
         <v>12</v>
       </c>
-      <c r="P9" s="36"/>
-      <c r="Q9" s="36"/>
-      <c r="R9" s="36"/>
-      <c r="S9" s="36"/>
-      <c r="T9" s="36"/>
-      <c r="U9" s="35" t="s">
+      <c r="P9" s="37"/>
+      <c r="Q9" s="37"/>
+      <c r="R9" s="37"/>
+      <c r="S9" s="37"/>
+      <c r="T9" s="37"/>
+      <c r="U9" s="40" t="s">
         <v>23</v>
       </c>
-      <c r="V9" s="36"/>
-      <c r="W9" s="36"/>
-      <c r="X9" s="36"/>
-      <c r="Y9" s="36"/>
-      <c r="Z9" s="36"/>
-      <c r="AA9" s="36"/>
-      <c r="AB9" s="36"/>
-      <c r="AC9" s="36"/>
+      <c r="V9" s="37"/>
+      <c r="W9" s="37"/>
+      <c r="X9" s="37"/>
+      <c r="Y9" s="37"/>
+      <c r="Z9" s="37"/>
+      <c r="AA9" s="37"/>
+      <c r="AB9" s="37"/>
+      <c r="AC9" s="37"/>
       <c r="AD9" s="27" t="s">
         <v>26</v>
       </c>
@@ -1121,7 +1117,7 @@
       <c r="AI9" s="13"/>
       <c r="AK9" s="16"/>
     </row>
-    <row r="10" spans="1:40" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:40" ht="14.25" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A10" s="26" t="s">
         <v>14</v>
       </c>
@@ -1129,36 +1125,36 @@
       <c r="C10" s="24"/>
       <c r="D10" s="24"/>
       <c r="E10" s="24"/>
-      <c r="F10" s="28"/>
-      <c r="G10" s="24"/>
-      <c r="H10" s="24"/>
-      <c r="I10" s="35" t="s">
+      <c r="F10" s="40" t="s">
         <v>19</v>
       </c>
-      <c r="J10" s="36"/>
-      <c r="K10" s="36"/>
-      <c r="L10" s="36"/>
-      <c r="M10" s="36"/>
-      <c r="N10" s="36"/>
-      <c r="O10" s="35" t="s">
+      <c r="G10" s="40"/>
+      <c r="H10" s="40"/>
+      <c r="I10" s="40"/>
+      <c r="J10" s="40"/>
+      <c r="K10" s="40"/>
+      <c r="L10" s="40"/>
+      <c r="M10" s="40"/>
+      <c r="N10" s="40"/>
+      <c r="O10" s="40" t="s">
         <v>18</v>
       </c>
-      <c r="P10" s="36"/>
-      <c r="Q10" s="36"/>
-      <c r="R10" s="36"/>
-      <c r="S10" s="36"/>
-      <c r="T10" s="36"/>
-      <c r="U10" s="36" t="s">
+      <c r="P10" s="37"/>
+      <c r="Q10" s="37"/>
+      <c r="R10" s="37"/>
+      <c r="S10" s="37"/>
+      <c r="T10" s="37"/>
+      <c r="U10" s="37" t="s">
         <v>12</v>
       </c>
-      <c r="V10" s="36"/>
-      <c r="W10" s="36"/>
-      <c r="X10" s="36"/>
-      <c r="Y10" s="36"/>
-      <c r="Z10" s="36"/>
-      <c r="AA10" s="36"/>
-      <c r="AB10" s="36"/>
-      <c r="AC10" s="36"/>
+      <c r="V10" s="37"/>
+      <c r="W10" s="37"/>
+      <c r="X10" s="37"/>
+      <c r="Y10" s="37"/>
+      <c r="Z10" s="37"/>
+      <c r="AA10" s="37"/>
+      <c r="AB10" s="37"/>
+      <c r="AC10" s="37"/>
       <c r="AD10" s="27" t="s">
         <v>27</v>
       </c>
@@ -1172,7 +1168,7 @@
       <c r="AM10" s="12"/>
       <c r="AN10" s="12"/>
     </row>
-    <row r="11" spans="1:40" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:40" ht="14.25" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A11" s="26" t="s">
         <v>15</v>
       </c>
@@ -1180,36 +1176,36 @@
       <c r="C11" s="24"/>
       <c r="D11" s="24"/>
       <c r="E11" s="24"/>
-      <c r="F11" s="28"/>
-      <c r="G11" s="24"/>
-      <c r="H11" s="24"/>
-      <c r="I11" s="35" t="s">
+      <c r="F11" s="40" t="s">
         <v>13</v>
       </c>
-      <c r="J11" s="36"/>
-      <c r="K11" s="36"/>
-      <c r="L11" s="36"/>
-      <c r="M11" s="36"/>
-      <c r="N11" s="36"/>
-      <c r="O11" s="35" t="s">
+      <c r="G11" s="40"/>
+      <c r="H11" s="40"/>
+      <c r="I11" s="40"/>
+      <c r="J11" s="40"/>
+      <c r="K11" s="40"/>
+      <c r="L11" s="40"/>
+      <c r="M11" s="40"/>
+      <c r="N11" s="40"/>
+      <c r="O11" s="40" t="s">
         <v>19</v>
       </c>
-      <c r="P11" s="36"/>
-      <c r="Q11" s="36"/>
-      <c r="R11" s="36"/>
-      <c r="S11" s="36"/>
-      <c r="T11" s="36"/>
-      <c r="U11" s="36" t="s">
+      <c r="P11" s="37"/>
+      <c r="Q11" s="37"/>
+      <c r="R11" s="37"/>
+      <c r="S11" s="37"/>
+      <c r="T11" s="37"/>
+      <c r="U11" s="37" t="s">
         <v>18</v>
       </c>
-      <c r="V11" s="36"/>
-      <c r="W11" s="36"/>
-      <c r="X11" s="36"/>
-      <c r="Y11" s="36"/>
-      <c r="Z11" s="36"/>
-      <c r="AA11" s="36"/>
-      <c r="AB11" s="36"/>
-      <c r="AC11" s="36"/>
+      <c r="V11" s="37"/>
+      <c r="W11" s="37"/>
+      <c r="X11" s="37"/>
+      <c r="Y11" s="37"/>
+      <c r="Z11" s="37"/>
+      <c r="AA11" s="37"/>
+      <c r="AB11" s="37"/>
+      <c r="AC11" s="37"/>
       <c r="AD11" s="27" t="s">
         <v>28</v>
       </c>
@@ -1220,7 +1216,7 @@
       <c r="AI11" s="13"/>
       <c r="AK11" s="14"/>
     </row>
-    <row r="12" spans="1:40" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:40" ht="14.25" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A12" s="26" t="s">
         <v>16</v>
       </c>
@@ -1228,36 +1224,36 @@
       <c r="C12" s="24"/>
       <c r="D12" s="24"/>
       <c r="E12" s="24"/>
-      <c r="F12" s="28"/>
-      <c r="G12" s="24"/>
-      <c r="H12" s="24"/>
-      <c r="I12" s="37" t="s">
+      <c r="F12" s="42" t="s">
         <v>21</v>
       </c>
-      <c r="J12" s="38"/>
-      <c r="K12" s="38"/>
-      <c r="L12" s="38"/>
-      <c r="M12" s="38"/>
-      <c r="N12" s="38"/>
-      <c r="O12" s="35" t="s">
+      <c r="G12" s="42"/>
+      <c r="H12" s="42"/>
+      <c r="I12" s="42"/>
+      <c r="J12" s="42"/>
+      <c r="K12" s="42"/>
+      <c r="L12" s="42"/>
+      <c r="M12" s="42"/>
+      <c r="N12" s="42"/>
+      <c r="O12" s="40" t="s">
         <v>13</v>
       </c>
-      <c r="P12" s="36"/>
-      <c r="Q12" s="36"/>
-      <c r="R12" s="36"/>
-      <c r="S12" s="36"/>
-      <c r="T12" s="36"/>
-      <c r="U12" s="36" t="s">
+      <c r="P12" s="37"/>
+      <c r="Q12" s="37"/>
+      <c r="R12" s="37"/>
+      <c r="S12" s="37"/>
+      <c r="T12" s="37"/>
+      <c r="U12" s="37" t="s">
         <v>19</v>
       </c>
-      <c r="V12" s="36"/>
-      <c r="W12" s="36"/>
-      <c r="X12" s="36"/>
-      <c r="Y12" s="36"/>
-      <c r="Z12" s="36"/>
-      <c r="AA12" s="36"/>
-      <c r="AB12" s="36"/>
-      <c r="AC12" s="36"/>
+      <c r="V12" s="37"/>
+      <c r="W12" s="37"/>
+      <c r="X12" s="37"/>
+      <c r="Y12" s="37"/>
+      <c r="Z12" s="37"/>
+      <c r="AA12" s="37"/>
+      <c r="AB12" s="37"/>
+      <c r="AC12" s="37"/>
       <c r="AD12" s="27" t="s">
         <v>29</v>
       </c>
@@ -1268,7 +1264,7 @@
       <c r="AI12" s="13"/>
       <c r="AK12" s="14"/>
     </row>
-    <row r="13" spans="1:40" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:40" ht="14.25" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A13" s="26" t="s">
         <v>17</v>
       </c>
@@ -1276,36 +1272,36 @@
       <c r="C13" s="24"/>
       <c r="D13" s="24"/>
       <c r="E13" s="24"/>
-      <c r="F13" s="28"/>
-      <c r="G13" s="24"/>
-      <c r="H13" s="24"/>
-      <c r="I13" s="37" t="s">
+      <c r="F13" s="42" t="s">
         <v>22</v>
       </c>
-      <c r="J13" s="38"/>
-      <c r="K13" s="38"/>
-      <c r="L13" s="38"/>
-      <c r="M13" s="38"/>
-      <c r="N13" s="38"/>
-      <c r="O13" s="35" t="s">
+      <c r="G13" s="42"/>
+      <c r="H13" s="42"/>
+      <c r="I13" s="42"/>
+      <c r="J13" s="42"/>
+      <c r="K13" s="42"/>
+      <c r="L13" s="42"/>
+      <c r="M13" s="42"/>
+      <c r="N13" s="42"/>
+      <c r="O13" s="40" t="s">
         <v>21</v>
       </c>
-      <c r="P13" s="36"/>
-      <c r="Q13" s="36"/>
-      <c r="R13" s="36"/>
-      <c r="S13" s="36"/>
-      <c r="T13" s="36"/>
-      <c r="U13" s="36" t="s">
+      <c r="P13" s="37"/>
+      <c r="Q13" s="37"/>
+      <c r="R13" s="37"/>
+      <c r="S13" s="37"/>
+      <c r="T13" s="37"/>
+      <c r="U13" s="37" t="s">
         <v>13</v>
       </c>
-      <c r="V13" s="36"/>
-      <c r="W13" s="36"/>
-      <c r="X13" s="36"/>
-      <c r="Y13" s="36"/>
-      <c r="Z13" s="36"/>
-      <c r="AA13" s="36"/>
-      <c r="AB13" s="36"/>
-      <c r="AC13" s="36"/>
+      <c r="V13" s="37"/>
+      <c r="W13" s="37"/>
+      <c r="X13" s="37"/>
+      <c r="Y13" s="37"/>
+      <c r="Z13" s="37"/>
+      <c r="AA13" s="37"/>
+      <c r="AB13" s="37"/>
+      <c r="AC13" s="37"/>
       <c r="AD13" s="27" t="s">
         <v>30</v>
       </c>
@@ -1319,7 +1315,7 @@
       <c r="AM13" s="12"/>
       <c r="AN13" s="12"/>
     </row>
-    <row r="14" spans="1:40" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:40" ht="14.25" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A14" s="26" t="s">
         <v>0</v>
       </c>
@@ -1327,73 +1323,73 @@
       <c r="C14" s="24"/>
       <c r="D14" s="24"/>
       <c r="E14" s="24"/>
-      <c r="F14" s="28"/>
-      <c r="G14" s="24"/>
-      <c r="H14" s="24"/>
-      <c r="I14" s="35" t="s">
+      <c r="F14" s="40" t="s">
         <v>20</v>
       </c>
-      <c r="J14" s="36"/>
-      <c r="K14" s="36"/>
-      <c r="L14" s="36"/>
-      <c r="M14" s="36"/>
-      <c r="N14" s="36"/>
-      <c r="O14" s="35" t="s">
+      <c r="G14" s="40"/>
+      <c r="H14" s="40"/>
+      <c r="I14" s="40"/>
+      <c r="J14" s="40"/>
+      <c r="K14" s="40"/>
+      <c r="L14" s="40"/>
+      <c r="M14" s="40"/>
+      <c r="N14" s="40"/>
+      <c r="O14" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="P14" s="36"/>
-      <c r="Q14" s="36"/>
-      <c r="R14" s="36"/>
-      <c r="S14" s="36"/>
-      <c r="T14" s="36"/>
-      <c r="U14" s="36" t="s">
+      <c r="P14" s="37"/>
+      <c r="Q14" s="37"/>
+      <c r="R14" s="37"/>
+      <c r="S14" s="37"/>
+      <c r="T14" s="37"/>
+      <c r="U14" s="37" t="s">
         <v>21</v>
       </c>
-      <c r="V14" s="36"/>
-      <c r="W14" s="36"/>
-      <c r="X14" s="36"/>
-      <c r="Y14" s="36"/>
-      <c r="Z14" s="36"/>
-      <c r="AA14" s="36"/>
-      <c r="AB14" s="36"/>
-      <c r="AC14" s="36"/>
+      <c r="V14" s="37"/>
+      <c r="W14" s="37"/>
+      <c r="X14" s="37"/>
+      <c r="Y14" s="37"/>
+      <c r="Z14" s="37"/>
+      <c r="AA14" s="37"/>
+      <c r="AB14" s="37"/>
+      <c r="AC14" s="37"/>
       <c r="AD14" s="25"/>
     </row>
     <row r="15" spans="1:40" x14ac:dyDescent="0.4">
-      <c r="A15" s="29" t="s">
+      <c r="A15" s="28" t="s">
         <v>34</v>
       </c>
-      <c r="B15" s="29"/>
-      <c r="C15" s="30"/>
-      <c r="D15" s="30"/>
-      <c r="E15" s="30"/>
-      <c r="F15" s="31"/>
+      <c r="B15" s="28"/>
+      <c r="C15" s="29"/>
+      <c r="D15" s="29"/>
+      <c r="E15" s="29"/>
+      <c r="F15" s="30"/>
       <c r="AL15" s="12"/>
       <c r="AM15" s="12"/>
       <c r="AN15" s="12"/>
     </row>
     <row r="16" spans="1:40" x14ac:dyDescent="0.4">
-      <c r="A16" s="32" t="s">
+      <c r="A16" s="31" t="s">
         <v>24</v>
       </c>
-      <c r="B16" s="32"/>
-      <c r="C16" s="30"/>
-      <c r="D16" s="30"/>
-      <c r="E16" s="30"/>
-      <c r="F16" s="31"/>
+      <c r="B16" s="31"/>
+      <c r="C16" s="29"/>
+      <c r="D16" s="29"/>
+      <c r="E16" s="29"/>
+      <c r="F16" s="30"/>
     </row>
     <row r="17" spans="1:40" x14ac:dyDescent="0.4">
-      <c r="A17" s="33" t="s">
+      <c r="A17" s="32" t="s">
         <v>1</v>
       </c>
-      <c r="B17" s="33"/>
-      <c r="C17" s="34">
+      <c r="B17" s="32"/>
+      <c r="C17" s="41">
         <f>55/15</f>
         <v>3.6666666666666665</v>
       </c>
-      <c r="D17" s="34"/>
-      <c r="E17" s="34"/>
-      <c r="F17" s="31" t="s">
+      <c r="D17" s="41"/>
+      <c r="E17" s="41"/>
+      <c r="F17" s="30" t="s">
         <v>25</v>
       </c>
       <c r="AL17" s="12"/>
@@ -1401,83 +1397,83 @@
       <c r="AN17" s="12"/>
     </row>
     <row r="18" spans="1:40" x14ac:dyDescent="0.4">
-      <c r="A18" s="33" t="s">
+      <c r="A18" s="32" t="s">
         <v>14</v>
       </c>
-      <c r="B18" s="33"/>
-      <c r="C18" s="34">
+      <c r="B18" s="32"/>
+      <c r="C18" s="41">
         <f>65/15</f>
         <v>4.333333333333333</v>
       </c>
-      <c r="D18" s="34"/>
-      <c r="E18" s="34"/>
-      <c r="F18" s="31" t="s">
+      <c r="D18" s="41"/>
+      <c r="E18" s="41"/>
+      <c r="F18" s="30" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="19" spans="1:40" x14ac:dyDescent="0.4">
-      <c r="A19" s="33" t="s">
+      <c r="A19" s="32" t="s">
         <v>15</v>
       </c>
-      <c r="B19" s="33"/>
-      <c r="C19" s="34">
+      <c r="B19" s="32"/>
+      <c r="C19" s="41">
         <f>75/15</f>
         <v>5</v>
       </c>
-      <c r="D19" s="34"/>
-      <c r="E19" s="34"/>
-      <c r="F19" s="31"/>
+      <c r="D19" s="41"/>
+      <c r="E19" s="41"/>
+      <c r="F19" s="30"/>
       <c r="O19" s="14"/>
       <c r="P19" s="14"/>
       <c r="Q19" s="14"/>
       <c r="R19" s="14"/>
     </row>
     <row r="20" spans="1:40" x14ac:dyDescent="0.4">
-      <c r="A20" s="33" t="s">
+      <c r="A20" s="32" t="s">
         <v>16</v>
       </c>
-      <c r="B20" s="33"/>
-      <c r="C20" s="34">
+      <c r="B20" s="32"/>
+      <c r="C20" s="41">
         <f>85/15</f>
         <v>5.666666666666667</v>
       </c>
-      <c r="D20" s="34"/>
-      <c r="E20" s="34"/>
-      <c r="F20" s="31"/>
+      <c r="D20" s="41"/>
+      <c r="E20" s="41"/>
+      <c r="F20" s="30"/>
       <c r="O20" s="14"/>
       <c r="P20" s="14"/>
       <c r="Q20" s="14"/>
       <c r="R20" s="14"/>
     </row>
     <row r="21" spans="1:40" x14ac:dyDescent="0.4">
-      <c r="A21" s="33" t="s">
+      <c r="A21" s="32" t="s">
         <v>17</v>
       </c>
-      <c r="B21" s="33"/>
-      <c r="C21" s="34">
+      <c r="B21" s="32"/>
+      <c r="C21" s="41">
         <f>95/15</f>
         <v>6.333333333333333</v>
       </c>
-      <c r="D21" s="34"/>
-      <c r="E21" s="34"/>
-      <c r="F21" s="31"/>
+      <c r="D21" s="41"/>
+      <c r="E21" s="41"/>
+      <c r="F21" s="30"/>
       <c r="O21" s="14"/>
       <c r="P21" s="14"/>
       <c r="Q21" s="14"/>
       <c r="R21" s="14"/>
     </row>
     <row r="22" spans="1:40" x14ac:dyDescent="0.4">
-      <c r="A22" s="33" t="s">
+      <c r="A22" s="32" t="s">
         <v>0</v>
       </c>
-      <c r="B22" s="33"/>
-      <c r="C22" s="34">
+      <c r="B22" s="32"/>
+      <c r="C22" s="41">
         <f>105/15</f>
         <v>7</v>
       </c>
-      <c r="D22" s="34"/>
-      <c r="E22" s="34"/>
-      <c r="F22" s="31"/>
+      <c r="D22" s="41"/>
+      <c r="E22" s="41"/>
+      <c r="F22" s="30"/>
       <c r="J22" s="5"/>
       <c r="K22" s="5"/>
       <c r="L22" s="5"/>
@@ -1595,6 +1591,42 @@
     </row>
   </sheetData>
   <mergeCells count="52">
+    <mergeCell ref="C22:E22"/>
+    <mergeCell ref="O9:T9"/>
+    <mergeCell ref="O10:T10"/>
+    <mergeCell ref="C21:E21"/>
+    <mergeCell ref="C17:E17"/>
+    <mergeCell ref="C18:E18"/>
+    <mergeCell ref="C19:E19"/>
+    <mergeCell ref="C20:E20"/>
+    <mergeCell ref="F9:N9"/>
+    <mergeCell ref="F10:N10"/>
+    <mergeCell ref="F11:N11"/>
+    <mergeCell ref="F12:N12"/>
+    <mergeCell ref="F13:N13"/>
+    <mergeCell ref="F14:N14"/>
+    <mergeCell ref="U13:AC13"/>
+    <mergeCell ref="AD7:AI7"/>
+    <mergeCell ref="AD6:AI6"/>
+    <mergeCell ref="AD5:AI5"/>
+    <mergeCell ref="X7:AC7"/>
+    <mergeCell ref="U9:AC9"/>
+    <mergeCell ref="U14:AC14"/>
+    <mergeCell ref="X5:AC5"/>
+    <mergeCell ref="S7:W7"/>
+    <mergeCell ref="S6:W6"/>
+    <mergeCell ref="O11:T11"/>
+    <mergeCell ref="O12:T12"/>
+    <mergeCell ref="O13:T13"/>
+    <mergeCell ref="O14:T14"/>
+    <mergeCell ref="S5:W5"/>
+    <mergeCell ref="M7:R7"/>
+    <mergeCell ref="M6:R6"/>
+    <mergeCell ref="M5:R5"/>
+    <mergeCell ref="U10:AC10"/>
+    <mergeCell ref="U11:AC11"/>
+    <mergeCell ref="U12:AC12"/>
+    <mergeCell ref="X6:AC6"/>
     <mergeCell ref="C7:E7"/>
     <mergeCell ref="C5:E5"/>
     <mergeCell ref="AD3:AI3"/>
@@ -1611,42 +1643,6 @@
     <mergeCell ref="F7:H7"/>
     <mergeCell ref="F6:H6"/>
     <mergeCell ref="F5:H5"/>
-    <mergeCell ref="U14:AC14"/>
-    <mergeCell ref="X5:AC5"/>
-    <mergeCell ref="S7:W7"/>
-    <mergeCell ref="S6:W6"/>
-    <mergeCell ref="O11:T11"/>
-    <mergeCell ref="O12:T12"/>
-    <mergeCell ref="O13:T13"/>
-    <mergeCell ref="O14:T14"/>
-    <mergeCell ref="S5:W5"/>
-    <mergeCell ref="M7:R7"/>
-    <mergeCell ref="M6:R6"/>
-    <mergeCell ref="M5:R5"/>
-    <mergeCell ref="U10:AC10"/>
-    <mergeCell ref="U11:AC11"/>
-    <mergeCell ref="U12:AC12"/>
-    <mergeCell ref="X6:AC6"/>
-    <mergeCell ref="U13:AC13"/>
-    <mergeCell ref="AD7:AI7"/>
-    <mergeCell ref="AD6:AI6"/>
-    <mergeCell ref="AD5:AI5"/>
-    <mergeCell ref="X7:AC7"/>
-    <mergeCell ref="U9:AC9"/>
-    <mergeCell ref="O9:T9"/>
-    <mergeCell ref="O10:T10"/>
-    <mergeCell ref="C21:E21"/>
-    <mergeCell ref="C17:E17"/>
-    <mergeCell ref="C18:E18"/>
-    <mergeCell ref="C19:E19"/>
-    <mergeCell ref="C20:E20"/>
-    <mergeCell ref="C22:E22"/>
-    <mergeCell ref="I9:N9"/>
-    <mergeCell ref="I10:N10"/>
-    <mergeCell ref="I11:N11"/>
-    <mergeCell ref="I12:N12"/>
-    <mergeCell ref="I13:N13"/>
-    <mergeCell ref="I14:N14"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="A1" r:id="rId1" xr:uid="{262308BA-9AEC-44C1-B6C0-92E820B5EA69}"/>

</xml_diff>